<commit_message>
fix(platform-audit): patch 5 enterprise audit issues - mask bot token, unmerge 114 cells in AI audit, add internal navbars, expand formulas to 50k rows, add capacity watchdog
</commit_message>
<xml_diff>
--- a/web/RevOps_Platform_Demo_Sample.xlsx
+++ b/web/RevOps_Platform_Demo_Sample.xlsx
@@ -26,7 +26,7 @@
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="0.0 &quot;ср.&quot;"/>
   </numFmts>
-  <fonts count="27">
+  <fonts count="28">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -189,6 +189,12 @@
       <color rgb="001E293B"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="0038BDF8"/>
+      <sz val="9"/>
+    </font>
   </fonts>
   <fills count="13">
     <fill>
@@ -264,7 +270,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -300,11 +306,93 @@
         <color rgb="000F172A"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom style="double">
+        <color rgb="000F172A"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom style="double">
+        <color rgb="000F172A"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="001E293B"/>
+      </left>
+      <right style="thin">
+        <color rgb="001E293B"/>
+      </right>
+      <top style="thin">
+        <color rgb="00334155"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00334155"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="98">
+  <cellXfs count="134">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -562,6 +650,110 @@
     </xf>
     <xf numFmtId="0" fontId="26" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="2" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="2" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="2" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -948,50 +1140,46 @@
           <t>⚡ ЭКСПРЕСС-КАЛЬКУЛЯТОР УПУЩЕННОЙ ПРИБЫЛИ ОП (ДИАГНОСТИКА ЗА 30 СЕКУНД)</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
-      <c r="I1" s="2" t="n"/>
     </row>
     <row r="2" ht="24" customHeight="1">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>⚡ Экспресс-Калькулятор</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>📋 Пульт РОПа (15 мин)</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="n"/>
-      <c r="D2" s="4" t="inlineStr">
-        <is>
-          <t>🎙️ ИИ-Аудит звонков</t>
-        </is>
-      </c>
-      <c r="E2" s="4" t="n"/>
-      <c r="F2" s="4" t="inlineStr">
-        <is>
-          <t>💸 7 Грехов (Диагностика)</t>
-        </is>
-      </c>
-      <c r="G2" s="4" t="inlineStr">
-        <is>
-          <t>📄 Executive One-Pager</t>
-        </is>
-      </c>
-      <c r="H2" s="4" t="n"/>
-      <c r="I2" s="4" t="inlineStr">
-        <is>
-          <t>🔐 152-ФЗ Безопасность</t>
-        </is>
-      </c>
-    </row>
+      <c r="A2" s="133">
+        <f>HYPERLINK("#'📄 Executive_OnePager'!A1", "📄 1. One-Pager")</f>
+        <v/>
+      </c>
+      <c r="B2" s="133">
+        <f>HYPERLINK("#'⚡ Пульс_Компании'!A1", "⚡ 2. Пульс компании")</f>
+        <v/>
+      </c>
+      <c r="C2" s="133">
+        <f>HYPERLINK("#'📋 Пульт_РОПа_15_Минут'!A1", "📋 3. Пульт РОПа")</f>
+        <v/>
+      </c>
+      <c r="D2" s="133">
+        <f>HYPERLINK("#'💸 Диагностика_Утечек_ОП'!A1", "💸 4. 7 Грехов ОП")</f>
+        <v/>
+      </c>
+      <c r="E2" s="133">
+        <f>HYPERLINK("#'🎯 Action_Center'!A1", "🎯 5. Action Center")</f>
+        <v/>
+      </c>
+      <c r="F2" s="133">
+        <f>HYPERLINK("#'🎙️ ИИ_Аудит'!A1", "🎙️ 6. ИИ-Аудит")</f>
+        <v/>
+      </c>
+      <c r="G2" s="133">
+        <f>HYPERLINK("#'⚡ Экспресс_Калькулятор_3_Цифры'!A1", "⚡ 7. Экспресс 3 цифры")</f>
+        <v/>
+      </c>
+      <c r="H2" s="133">
+        <f>HYPERLINK("#'🧪 QA_Suite'!A1", "🧪 8. QA Suite")</f>
+        <v/>
+      </c>
+      <c r="I2" s="133">
+        <f>HYPERLINK("#'⚙️ Настройки'!A1", "⚙️ 9. Настройки")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4" ht="24" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
         <is>
@@ -1008,7 +1196,6 @@
           <t>Категория капитала</t>
         </is>
       </c>
-      <c r="H4" s="7" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
@@ -1112,46 +1299,56 @@
         <v/>
       </c>
     </row>
+    <row r="9"/>
     <row r="10" ht="22" customHeight="1">
       <c r="A10" s="17" t="inlineStr">
         <is>
           <t>🔴 ВЫЯВЛЕННЫЙ РИСК ПОТЕРЬ</t>
         </is>
       </c>
+      <c r="B10" s="98" t="n"/>
       <c r="C10" s="18" t="inlineStr">
         <is>
           <t>🟢 КОНСЕРВАТИВНЫЙ (+15%)</t>
         </is>
       </c>
+      <c r="D10" s="98" t="n"/>
       <c r="E10" s="19" t="inlineStr">
         <is>
           <t>🚀 БАЗОВЫЙ ПЛАН (+30%)</t>
         </is>
       </c>
+      <c r="F10" s="98" t="n"/>
       <c r="G10" s="20" t="inlineStr">
         <is>
           <t>⭐ ОПТИМИСТИЧНЫЙ (+50%)</t>
         </is>
       </c>
+      <c r="H10" s="98" t="n"/>
     </row>
     <row r="11" ht="32" customHeight="1">
       <c r="A11" s="21">
         <f>H6</f>
         <v/>
       </c>
+      <c r="B11" s="98" t="n"/>
       <c r="C11" s="22">
         <f>H5*1.0945</f>
         <v/>
       </c>
+      <c r="D11" s="98" t="n"/>
       <c r="E11" s="23">
         <f>H5*1.189</f>
         <v/>
       </c>
+      <c r="F11" s="98" t="n"/>
       <c r="G11" s="24">
         <f>H5*1.315</f>
         <v/>
       </c>
-    </row>
+      <c r="H11" s="98" t="n"/>
+    </row>
+    <row r="12"/>
     <row r="13" ht="24" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
         <is>
@@ -1337,20 +1534,13 @@
         <v/>
       </c>
     </row>
+    <row r="20"/>
     <row r="21" ht="28" customHeight="1">
       <c r="A21" s="33" t="inlineStr">
         <is>
           <t>🎁 СЛЕДУЮЩИЙ ШАГ: БЕСПЛАТНЫЙ ТЕСТ-ДРАЙВ НА 3 ВАШИХ ЗВОНКАХ</t>
         </is>
       </c>
-      <c r="B21" s="33" t="n"/>
-      <c r="C21" s="33" t="n"/>
-      <c r="D21" s="33" t="n"/>
-      <c r="E21" s="33" t="n"/>
-      <c r="F21" s="33" t="n"/>
-      <c r="G21" s="33" t="n"/>
-      <c r="H21" s="33" t="n"/>
-      <c r="I21" s="33" t="n"/>
     </row>
     <row r="22" ht="24" customHeight="1">
       <c r="A22" s="34" t="inlineStr">
@@ -1358,14 +1548,6 @@
           <t>Хотите проверить эту математику на реальных данных вашей компании за 15 минут?</t>
         </is>
       </c>
-      <c r="B22" s="34" t="n"/>
-      <c r="C22" s="34" t="n"/>
-      <c r="D22" s="34" t="n"/>
-      <c r="E22" s="34" t="n"/>
-      <c r="F22" s="34" t="n"/>
-      <c r="G22" s="34" t="n"/>
-      <c r="H22" s="34" t="n"/>
-      <c r="I22" s="34" t="n"/>
     </row>
     <row r="23" ht="24" customHeight="1">
       <c r="A23" s="35" t="inlineStr">
@@ -1373,14 +1555,6 @@
           <t>👉 Отправьте 3 аудиозаписи любых вчерашних звонков ваших менеджеров в Telegram бот.</t>
         </is>
       </c>
-      <c r="B23" s="35" t="n"/>
-      <c r="C23" s="35" t="n"/>
-      <c r="D23" s="35" t="n"/>
-      <c r="E23" s="35" t="n"/>
-      <c r="F23" s="35" t="n"/>
-      <c r="G23" s="35" t="n"/>
-      <c r="H23" s="35" t="n"/>
-      <c r="I23" s="35" t="n"/>
     </row>
     <row r="24" ht="24" customHeight="1">
       <c r="A24" s="35" t="inlineStr">
@@ -1388,14 +1562,6 @@
           <t>ИИ бесплатно разберет их по 13 критериям, покажет ошибки речи и рассчитает точную сумму под угрозой слива.</t>
         </is>
       </c>
-      <c r="B24" s="35" t="n"/>
-      <c r="C24" s="35" t="n"/>
-      <c r="D24" s="35" t="n"/>
-      <c r="E24" s="35" t="n"/>
-      <c r="F24" s="35" t="n"/>
-      <c r="G24" s="35" t="n"/>
-      <c r="H24" s="35" t="n"/>
-      <c r="I24" s="35" t="n"/>
     </row>
     <row r="25" ht="32" customHeight="1">
       <c r="A25" s="36" t="inlineStr">
@@ -1403,14 +1569,6 @@
           <t>🚀 ЗАПУСТИТЬ БЕСПЛАТНЫЙ ТЕСТ-ДРАЙВ: @RevOps_Super_Audit_Bot (https://t.me/RevOps_Super_Audit_Bot)</t>
         </is>
       </c>
-      <c r="B25" s="36" t="n"/>
-      <c r="C25" s="36" t="n"/>
-      <c r="D25" s="36" t="n"/>
-      <c r="E25" s="36" t="n"/>
-      <c r="F25" s="36" t="n"/>
-      <c r="G25" s="36" t="n"/>
-      <c r="H25" s="36" t="n"/>
-      <c r="I25" s="36" t="n"/>
     </row>
     <row r="26" ht="24" customHeight="1">
       <c r="A26" s="37" t="inlineStr">
@@ -1418,14 +1576,6 @@
           <t>Нужен комплексный аудит отдела продаж? 👉 Экономика спринта оптимизации (450 000 ₽) на вкладке «4. 7 Грехов ОП»</t>
         </is>
       </c>
-      <c r="B26" s="37" t="n"/>
-      <c r="C26" s="37" t="n"/>
-      <c r="D26" s="37" t="n"/>
-      <c r="E26" s="37" t="n"/>
-      <c r="F26" s="37" t="n"/>
-      <c r="G26" s="37" t="n"/>
-      <c r="H26" s="37" t="n"/>
-      <c r="I26" s="37" t="n"/>
     </row>
     <row r="27" ht="24" customHeight="1">
       <c r="A27" s="38" t="inlineStr">
@@ -1433,28 +1583,17 @@
           <t>🔒 Конфиденциально • Без передачи персональных данных • Экспресс-разбор за 15 минут (152-ФЗ РФ)</t>
         </is>
       </c>
-      <c r="B27" s="38" t="n"/>
-      <c r="C27" s="38" t="n"/>
-      <c r="D27" s="38" t="n"/>
-      <c r="E27" s="38" t="n"/>
-      <c r="F27" s="38" t="n"/>
-      <c r="G27" s="38" t="n"/>
-      <c r="H27" s="38" t="n"/>
-      <c r="I27" s="38" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="23">
+  <mergeCells count="20">
     <mergeCell ref="A25:I25"/>
-    <mergeCell ref="G2:H2"/>
     <mergeCell ref="A11:B11"/>
     <mergeCell ref="G11:H11"/>
     <mergeCell ref="A27:I27"/>
     <mergeCell ref="A26:I26"/>
     <mergeCell ref="A21:I21"/>
     <mergeCell ref="C4:D4"/>
-    <mergeCell ref="B2:C2"/>
     <mergeCell ref="C10:D10"/>
-    <mergeCell ref="D2:E2"/>
     <mergeCell ref="E10:F10"/>
     <mergeCell ref="G10:H10"/>
     <mergeCell ref="A23:I23"/>
@@ -1486,7 +1625,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1505,55 +1644,53 @@
           <t>📋 СТРАТЕГИЧЕСКИЙ ПУЛЬТ СОБСТВЕННИКА: «5 РЕШЕНИЙ МЕСЯЦА»</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
     </row>
     <row r="2" ht="24" customHeight="1">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>⚡ Экспресс-Калькулятор</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="n"/>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>📋 Пульт РОПа</t>
-        </is>
-      </c>
-      <c r="D2" s="4" t="inlineStr">
-        <is>
-          <t>🎙️ ИИ-Аудит</t>
-        </is>
-      </c>
-      <c r="E2" s="4" t="inlineStr">
-        <is>
-          <t>💸 7 Грехов ОП</t>
-        </is>
-      </c>
-      <c r="F2" s="4" t="inlineStr">
-        <is>
-          <t>📄 One-Pager</t>
-        </is>
-      </c>
-      <c r="G2" s="4" t="inlineStr">
-        <is>
-          <t>🔐 152-ФЗ Безопасность</t>
-        </is>
-      </c>
-      <c r="H2" s="4" t="n"/>
-    </row>
+      <c r="A2" s="133">
+        <f>HYPERLINK("#'📄 Executive_OnePager'!A1", "📄 1. One-Pager")</f>
+        <v/>
+      </c>
+      <c r="B2" s="133">
+        <f>HYPERLINK("#'⚡ Пульс_Компании'!A1", "⚡ 2. Пульс компании")</f>
+        <v/>
+      </c>
+      <c r="C2" s="133">
+        <f>HYPERLINK("#'📋 Пульт_РОПа_15_Минут'!A1", "📋 3. Пульт РОПа")</f>
+        <v/>
+      </c>
+      <c r="D2" s="133">
+        <f>HYPERLINK("#'💸 Диагностика_Утечек_ОП'!A1", "💸 4. 7 Грехов ОП")</f>
+        <v/>
+      </c>
+      <c r="E2" s="133">
+        <f>HYPERLINK("#'🎯 Action_Center'!A1", "🎯 5. Action Center")</f>
+        <v/>
+      </c>
+      <c r="F2" s="133">
+        <f>HYPERLINK("#'🎙️ ИИ_Аудит'!A1", "🎙️ 6. ИИ-Аудит")</f>
+        <v/>
+      </c>
+      <c r="G2" s="133">
+        <f>HYPERLINK("#'⚡ Экспресс_Калькулятор_3_Цифры'!A1", "⚡ 7. Экспресс 3 цифры")</f>
+        <v/>
+      </c>
+      <c r="H2" s="133">
+        <f>HYPERLINK("#'🧪 QA_Suite'!A1", "🧪 8. QA Suite")</f>
+        <v/>
+      </c>
+      <c r="I2" s="133">
+        <f>HYPERLINK("#'⚙️ Настройки'!A1", "⚙️ 9. Настройки")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="39" t="inlineStr">
         <is>
           <t>Звонков за вчера</t>
         </is>
       </c>
-      <c r="B4" s="39" t="n"/>
+      <c r="B4" s="98" t="n"/>
       <c r="C4" s="40" t="inlineStr">
         <is>
           <t>Диалогов с браком (&lt;9)</t>
@@ -1574,14 +1711,14 @@
           <t>Статус дня для РОПа</t>
         </is>
       </c>
-      <c r="G4" s="40" t="n"/>
-      <c r="H4" s="40" t="n"/>
+      <c r="G4" s="99" t="n"/>
+      <c r="H4" s="98" t="n"/>
     </row>
     <row r="5" ht="32" customHeight="1">
       <c r="A5" s="41" t="n">
         <v>6</v>
       </c>
-      <c r="B5" s="41" t="n"/>
+      <c r="B5" s="98" t="n"/>
       <c r="C5" s="42" t="n">
         <v>2</v>
       </c>
@@ -1596,9 +1733,10 @@
           <t>🚨 ТРЕБУЕТСЯ 15 МИНУТ КОНТРОЛЯ РОПа</t>
         </is>
       </c>
-      <c r="G5" s="43" t="n"/>
-      <c r="H5" s="43" t="n"/>
-    </row>
+      <c r="G5" s="99" t="n"/>
+      <c r="H5" s="98" t="n"/>
+    </row>
+    <row r="6"/>
     <row r="7" ht="24" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
@@ -1867,6 +2005,8 @@
       </c>
       <c r="H14" s="29" t="n"/>
     </row>
+    <row r="15"/>
+    <row r="16"/>
     <row r="17" ht="24" customHeight="1">
       <c r="E17" s="50" t="inlineStr">
         <is>
@@ -1885,8 +2025,8 @@
           <t>Проверка ночного ИИ-аудита: 2 звонка с браком (&lt;9 баллов)</t>
         </is>
       </c>
-      <c r="G18" s="51" t="n"/>
-      <c r="H18" s="51" t="n"/>
+      <c r="G18" s="99" t="n"/>
+      <c r="H18" s="98" t="n"/>
     </row>
     <row r="19" ht="22" customHeight="1">
       <c r="E19" s="44" t="inlineStr">
@@ -1899,8 +2039,8 @@
           <t>Перехват сделки D-109 (600 т.р.) и звонок ЛПР до 12:00</t>
         </is>
       </c>
-      <c r="G19" s="51" t="n"/>
-      <c r="H19" s="51" t="n"/>
+      <c r="G19" s="99" t="n"/>
+      <c r="H19" s="98" t="n"/>
     </row>
     <row r="20" ht="22" customHeight="1">
       <c r="E20" s="44" t="inlineStr">
@@ -1913,8 +2053,8 @@
           <t>Согласование спецусловий по D-104 (850 т.р.)</t>
         </is>
       </c>
-      <c r="G20" s="51" t="n"/>
-      <c r="H20" s="51" t="n"/>
+      <c r="G20" s="99" t="n"/>
+      <c r="H20" s="98" t="n"/>
     </row>
     <row r="21" ht="22" customHeight="1">
       <c r="E21" s="44" t="inlineStr">
@@ -1927,8 +2067,8 @@
           <t>Делегирование 2 сделок с РОПа на свободного КАМа</t>
         </is>
       </c>
-      <c r="G21" s="51" t="n"/>
-      <c r="H21" s="51" t="n"/>
+      <c r="G21" s="99" t="n"/>
+      <c r="H21" s="98" t="n"/>
     </row>
     <row r="22" ht="22" customHeight="1">
       <c r="E22" s="18" t="inlineStr">
@@ -1941,19 +2081,17 @@
           <t>2 730 000 ₽ защищено от слива за 15 минут</t>
         </is>
       </c>
-      <c r="G22" s="51" t="n"/>
-      <c r="H22" s="51" t="n"/>
+      <c r="G22" s="99" t="n"/>
+      <c r="H22" s="98" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="14">
+  <mergeCells count="12">
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="F20:H20"/>
-    <mergeCell ref="A2:B2"/>
     <mergeCell ref="E17:H17"/>
     <mergeCell ref="F5:H5"/>
     <mergeCell ref="F19:H19"/>
     <mergeCell ref="A7:H7"/>
-    <mergeCell ref="G2:H2"/>
     <mergeCell ref="F18:H18"/>
     <mergeCell ref="F22:H22"/>
     <mergeCell ref="A5:B5"/>
@@ -1982,18 +2120,18 @@
   <dimension ref="A1:V60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="11" customWidth="1" min="10" max="10"/>
-    <col width="11" customWidth="1" min="11" max="11"/>
-    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
     <col width="11" customWidth="1" min="13" max="13"/>
     <col width="11" customWidth="1" min="14" max="14"/>
     <col width="11" customWidth="1" min="15" max="15"/>
@@ -2007,203 +2145,134 @@
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="100" t="inlineStr">
         <is>
           <t>🎙️ ИИ-СУПЕРВАЙЗЕР ЗВОНКОВ: РЕЧЕВАЯ АНАЛИТИКА 100% ДИАЛОГОВ (WHISPER LARGE V3 + LLM)</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
-      <c r="I1" s="2" t="n"/>
-      <c r="J1" s="2" t="n"/>
-      <c r="K1" s="2" t="n"/>
-      <c r="L1" s="2" t="n"/>
-      <c r="M1" s="2" t="n"/>
-      <c r="N1" s="2" t="n"/>
-      <c r="O1" s="2" t="n"/>
-      <c r="P1" s="2" t="n"/>
-      <c r="Q1" s="2" t="n"/>
-      <c r="R1" s="2" t="n"/>
-      <c r="S1" s="2" t="n"/>
-      <c r="T1" s="2" t="n"/>
-      <c r="U1" s="2" t="n"/>
-      <c r="V1" s="2" t="n"/>
     </row>
     <row r="2" ht="24" customHeight="1">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>⚡ Экспресс-Калькулятор</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="n"/>
-      <c r="C2" s="4" t="n"/>
-      <c r="D2" s="4" t="inlineStr">
-        <is>
-          <t>📋 Пульт РОПа (15 мин)</t>
-        </is>
-      </c>
-      <c r="E2" s="4" t="n"/>
-      <c r="F2" s="4" t="n"/>
-      <c r="G2" s="3" t="inlineStr">
-        <is>
-          <t>🎙️ ИИ-Аудит звонков</t>
-        </is>
-      </c>
-      <c r="H2" s="3" t="n"/>
-      <c r="I2" s="3" t="n"/>
-      <c r="J2" s="3" t="n"/>
-      <c r="K2" s="4" t="inlineStr">
+      <c r="A2" s="133">
+        <f>HYPERLINK("#'📄 Executive_OnePager'!A1", "📄 1. One-Pager")</f>
+        <v/>
+      </c>
+      <c r="B2" s="133">
+        <f>HYPERLINK("#'⚡ Пульс_Компании'!A1", "⚡ 2. Пульс компании")</f>
+        <v/>
+      </c>
+      <c r="C2" s="133">
+        <f>HYPERLINK("#'📋 Пульт_РОПа_15_Минут'!A1", "📋 3. Пульт РОПа")</f>
+        <v/>
+      </c>
+      <c r="D2" s="133">
+        <f>HYPERLINK("#'💸 Диагностика_Утечек_ОП'!A1", "💸 4. 7 Грехов ОП")</f>
+        <v/>
+      </c>
+      <c r="E2" s="133">
+        <f>HYPERLINK("#'🎯 Action_Center'!A1", "🎯 5. Action Center")</f>
+        <v/>
+      </c>
+      <c r="F2" s="133">
+        <f>HYPERLINK("#'🎙️ ИИ_Аудит'!A1", "🎙️ 6. ИИ-Аудит")</f>
+        <v/>
+      </c>
+      <c r="G2" s="133">
+        <f>HYPERLINK("#'⚡ Экспресс_Калькулятор_3_Цифры'!A1", "⚡ 7. Экспресс 3 цифры")</f>
+        <v/>
+      </c>
+      <c r="H2" s="133">
+        <f>HYPERLINK("#'🧪 QA_Suite'!A1", "🧪 8. QA Suite")</f>
+        <v/>
+      </c>
+      <c r="I2" s="133">
+        <f>HYPERLINK("#'⚙️ Настройки'!A1", "⚙️ 9. Настройки")</f>
+        <v/>
+      </c>
+      <c r="K2" s="102" t="inlineStr">
         <is>
           <t>💸 7 Грехов (Диагностика)</t>
         </is>
       </c>
-      <c r="L2" s="4" t="n"/>
-      <c r="M2" s="4" t="n"/>
-      <c r="N2" s="4" t="inlineStr">
+      <c r="N2" s="102" t="inlineStr">
         <is>
           <t>📄 Executive One-Pager</t>
         </is>
       </c>
-      <c r="O2" s="4" t="n"/>
-      <c r="P2" s="4" t="n"/>
       <c r="Q2" s="4" t="inlineStr">
         <is>
           <t>🔐 152-ФЗ Безопасность</t>
         </is>
       </c>
-      <c r="R2" s="4" t="n"/>
-      <c r="S2" s="4" t="n"/>
-      <c r="T2" s="4" t="n"/>
-      <c r="U2" s="4" t="n"/>
-      <c r="V2" s="4" t="n"/>
     </row>
     <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="39" t="inlineStr">
+      <c r="A3" s="95" t="inlineStr">
         <is>
           <t>Проанализировано звонков</t>
         </is>
       </c>
-      <c r="B3" s="39" t="n"/>
-      <c r="C3" s="53" t="inlineStr">
+      <c r="C3" s="96" t="inlineStr">
         <is>
           <t>Средний балл качества</t>
         </is>
       </c>
-      <c r="D3" s="53" t="n"/>
-      <c r="E3" s="54" t="inlineStr">
+      <c r="E3" s="103" t="inlineStr">
         <is>
           <t>Фиксация жесткого Next Step</t>
         </is>
       </c>
-      <c r="F3" s="54" t="n"/>
-      <c r="G3" s="40" t="inlineStr">
+      <c r="G3" s="84" t="inlineStr">
         <is>
           <t>Критический брак речи (&lt;9)</t>
         </is>
       </c>
-      <c r="H3" s="40" t="n"/>
-      <c r="I3" s="40" t="n"/>
-      <c r="J3" s="40" t="inlineStr">
+      <c r="J3" s="84" t="inlineStr">
         <is>
           <t>Выручка под угрозой слива</t>
         </is>
       </c>
-      <c r="K3" s="40" t="n"/>
-      <c r="L3" s="40" t="n"/>
-      <c r="M3" s="40" t="inlineStr">
+      <c r="M3" s="84" t="inlineStr">
         <is>
           <t>Вердикт ИИ-супервайзера</t>
         </is>
       </c>
-      <c r="N3" s="40" t="n"/>
-      <c r="O3" s="40" t="n"/>
-      <c r="P3" s="40" t="n"/>
-      <c r="Q3" s="40" t="n"/>
-      <c r="R3" s="40" t="n"/>
-      <c r="S3" s="40" t="n"/>
-      <c r="T3" s="40" t="n"/>
-      <c r="U3" s="40" t="n"/>
-      <c r="V3" s="40" t="n"/>
     </row>
     <row r="4" ht="32" customHeight="1">
-      <c r="A4" s="41" t="inlineStr">
+      <c r="A4" s="104" t="inlineStr">
         <is>
           <t>25 звонков / сут</t>
         </is>
       </c>
-      <c r="B4" s="41" t="n"/>
-      <c r="C4" s="55" t="inlineStr">
+      <c r="C4" s="105" t="inlineStr">
         <is>
           <t>8.9 из 13</t>
         </is>
       </c>
-      <c r="D4" s="55" t="n"/>
-      <c r="E4" s="56" t="inlineStr">
+      <c r="E4" s="106" t="inlineStr">
         <is>
           <t>60.0% (норма ≥85%)</t>
         </is>
       </c>
-      <c r="F4" s="56" t="n"/>
-      <c r="G4" s="42" t="inlineStr">
+      <c r="G4" s="107" t="inlineStr">
         <is>
           <t>6 диалогов</t>
         </is>
       </c>
-      <c r="H4" s="42" t="n"/>
-      <c r="I4" s="42" t="n"/>
-      <c r="J4" s="21" t="n">
+      <c r="J4" s="108" t="n">
         <v>2840000</v>
       </c>
-      <c r="K4" s="21" t="n"/>
-      <c r="L4" s="21" t="n"/>
-      <c r="M4" s="57" t="inlineStr">
+      <c r="M4" s="109" t="inlineStr">
         <is>
           <t>🚨 ВЫСОКИЙ РИСК СЛИВА VIP-КЛИЕНТОВ (ТРЕБУЕТСЯ ВМЕШАТЕЛЬСТВО РОПа)</t>
         </is>
       </c>
-      <c r="N4" s="57" t="n"/>
-      <c r="O4" s="57" t="n"/>
-      <c r="P4" s="57" t="n"/>
-      <c r="Q4" s="57" t="n"/>
-      <c r="R4" s="57" t="n"/>
-      <c r="S4" s="57" t="n"/>
-      <c r="T4" s="57" t="n"/>
-      <c r="U4" s="57" t="n"/>
-      <c r="V4" s="57" t="n"/>
     </row>
     <row r="5" ht="12" customHeight="1"/>
     <row r="6" ht="24" customHeight="1">
-      <c r="A6" s="58" t="inlineStr">
+      <c r="A6" s="110" t="inlineStr">
         <is>
           <t>👥 РЕЙТИНГ МЕНЕДЖЕРОВ ОП ПО КАЧЕСТВУ РЕЧИ (ЛИДЕРБОРД РОПа)</t>
         </is>
       </c>
-      <c r="B6" s="58" t="n"/>
-      <c r="C6" s="58" t="n"/>
-      <c r="D6" s="58" t="n"/>
-      <c r="E6" s="58" t="n"/>
-      <c r="F6" s="58" t="n"/>
-      <c r="G6" s="58" t="n"/>
-      <c r="H6" s="58" t="n"/>
-      <c r="I6" s="58" t="n"/>
-      <c r="J6" s="58" t="n"/>
-      <c r="K6" s="58" t="n"/>
-      <c r="L6" s="58" t="n"/>
-      <c r="M6" s="58" t="n"/>
-      <c r="N6" s="58" t="n"/>
-      <c r="O6" s="58" t="n"/>
-      <c r="P6" s="58" t="n"/>
-      <c r="Q6" s="58" t="n"/>
-      <c r="R6" s="58" t="n"/>
-      <c r="S6" s="58" t="n"/>
-      <c r="T6" s="58" t="n"/>
-      <c r="U6" s="58" t="n"/>
-      <c r="V6" s="58" t="n"/>
     </row>
     <row r="7" ht="32" customHeight="1">
       <c r="A7" s="59" t="inlineStr">
@@ -2251,45 +2320,33 @@
           <t>Грейд ИИ</t>
         </is>
       </c>
-      <c r="J7" s="25" t="inlineStr">
+      <c r="J7" s="59" t="inlineStr">
         <is>
           <t>Статус и рекомендация РОПу</t>
         </is>
       </c>
-      <c r="K7" s="25" t="n"/>
-      <c r="L7" s="25" t="n"/>
-      <c r="M7" s="25" t="n"/>
-      <c r="N7" s="25" t="n"/>
-      <c r="O7" s="25" t="n"/>
-      <c r="P7" s="25" t="n"/>
-      <c r="Q7" s="25" t="n"/>
-      <c r="R7" s="25" t="n"/>
-      <c r="S7" s="25" t="n"/>
-      <c r="T7" s="25" t="n"/>
-      <c r="U7" s="25" t="n"/>
-      <c r="V7" s="25" t="n"/>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="26" t="n">
-        <v>1</v>
-      </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="A8" s="111" t="n">
+        <v>1</v>
+      </c>
+      <c r="B8" s="74" t="inlineStr">
         <is>
           <t>Алексей Мельников</t>
         </is>
       </c>
-      <c r="C8" s="26" t="n">
+      <c r="C8" s="111" t="n">
         <v>6</v>
       </c>
-      <c r="D8" s="60" t="n">
+      <c r="D8" s="112" t="n">
         <v>12.2</v>
       </c>
-      <c r="E8" s="26" t="inlineStr">
+      <c r="E8" s="111" t="inlineStr">
         <is>
           <t>100.0%</t>
         </is>
       </c>
-      <c r="F8" s="26" t="inlineStr">
+      <c r="F8" s="111" t="inlineStr">
         <is>
           <t>48% / 52%</t>
         </is>
@@ -2300,330 +2357,237 @@
       <c r="H8" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="I8" s="18" t="inlineStr">
+      <c r="I8" s="113" t="inlineStr">
         <is>
           <t>⭐ А (Эталон)</t>
         </is>
       </c>
-      <c r="J8" s="61" t="inlineStr">
+      <c r="J8" s="27" t="inlineStr">
         <is>
           <t>Эталонный скрипт, рекомендован в базу знаний компании</t>
         </is>
       </c>
-      <c r="K8" s="61" t="n"/>
-      <c r="L8" s="61" t="n"/>
-      <c r="M8" s="61" t="n"/>
-      <c r="N8" s="61" t="n"/>
-      <c r="O8" s="61" t="n"/>
-      <c r="P8" s="61" t="n"/>
-      <c r="Q8" s="61" t="n"/>
-      <c r="R8" s="61" t="n"/>
-      <c r="S8" s="61" t="n"/>
-      <c r="T8" s="61" t="n"/>
-      <c r="U8" s="61" t="n"/>
-      <c r="V8" s="61" t="n"/>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="26" t="n">
+      <c r="A9" s="111" t="n">
         <v>2</v>
       </c>
-      <c r="B9" s="8" t="inlineStr">
+      <c r="B9" s="74" t="inlineStr">
         <is>
           <t>Елена Васильева</t>
         </is>
       </c>
-      <c r="C9" s="26" t="n">
+      <c r="C9" s="111" t="n">
         <v>5</v>
       </c>
-      <c r="D9" s="60" t="n">
+      <c r="D9" s="112" t="n">
         <v>10.8</v>
       </c>
-      <c r="E9" s="26" t="inlineStr">
+      <c r="E9" s="111" t="inlineStr">
         <is>
           <t>80.0%</t>
         </is>
       </c>
-      <c r="F9" s="26" t="inlineStr">
+      <c r="F9" s="111" t="inlineStr">
         <is>
           <t>51% / 49%</t>
         </is>
       </c>
-      <c r="G9" s="26" t="n">
-        <v>1</v>
-      </c>
-      <c r="H9" s="62" t="n">
+      <c r="G9" s="111" t="n">
+        <v>1</v>
+      </c>
+      <c r="H9" s="114" t="n">
         <v>160000</v>
       </c>
-      <c r="I9" s="18" t="inlineStr">
+      <c r="I9" s="113" t="inlineStr">
         <is>
           <t>🟢 B (Норма)</t>
         </is>
       </c>
-      <c r="J9" s="61" t="inlineStr">
+      <c r="J9" s="27" t="inlineStr">
         <is>
           <t>Высокая конверсия, мелкие замечания по регламенту встречи</t>
         </is>
       </c>
-      <c r="K9" s="61" t="n"/>
-      <c r="L9" s="61" t="n"/>
-      <c r="M9" s="61" t="n"/>
-      <c r="N9" s="61" t="n"/>
-      <c r="O9" s="61" t="n"/>
-      <c r="P9" s="61" t="n"/>
-      <c r="Q9" s="61" t="n"/>
-      <c r="R9" s="61" t="n"/>
-      <c r="S9" s="61" t="n"/>
-      <c r="T9" s="61" t="n"/>
-      <c r="U9" s="61" t="n"/>
-      <c r="V9" s="61" t="n"/>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="26" t="n">
+      <c r="A10" s="111" t="n">
         <v>3</v>
       </c>
-      <c r="B10" s="8" t="inlineStr">
+      <c r="B10" s="74" t="inlineStr">
         <is>
           <t>Анна Соколова</t>
         </is>
       </c>
-      <c r="C10" s="26" t="n">
+      <c r="C10" s="111" t="n">
         <v>5</v>
       </c>
-      <c r="D10" s="63" t="n">
+      <c r="D10" s="115" t="n">
         <v>8.4</v>
       </c>
-      <c r="E10" s="26" t="inlineStr">
+      <c r="E10" s="111" t="inlineStr">
         <is>
           <t>60.0%</t>
         </is>
       </c>
-      <c r="F10" s="26" t="inlineStr">
+      <c r="F10" s="111" t="inlineStr">
         <is>
           <t>58% / 42%</t>
         </is>
       </c>
-      <c r="G10" s="26" t="n">
+      <c r="G10" s="111" t="n">
         <v>2</v>
       </c>
-      <c r="H10" s="62" t="n">
+      <c r="H10" s="114" t="n">
         <v>480000</v>
       </c>
-      <c r="I10" s="20" t="inlineStr">
+      <c r="I10" s="116" t="inlineStr">
         <is>
           <t>🟡 C (Зона риска)</t>
         </is>
       </c>
-      <c r="J10" s="61" t="inlineStr">
+      <c r="J10" s="27" t="inlineStr">
         <is>
           <t>Забывает фиксировать дату звонка, требуется тренинг</t>
         </is>
       </c>
-      <c r="K10" s="61" t="n"/>
-      <c r="L10" s="61" t="n"/>
-      <c r="M10" s="61" t="n"/>
-      <c r="N10" s="61" t="n"/>
-      <c r="O10" s="61" t="n"/>
-      <c r="P10" s="61" t="n"/>
-      <c r="Q10" s="61" t="n"/>
-      <c r="R10" s="61" t="n"/>
-      <c r="S10" s="61" t="n"/>
-      <c r="T10" s="61" t="n"/>
-      <c r="U10" s="61" t="n"/>
-      <c r="V10" s="61" t="n"/>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="26" t="n">
+      <c r="A11" s="111" t="n">
         <v>4</v>
       </c>
-      <c r="B11" s="8" t="inlineStr">
+      <c r="B11" s="74" t="inlineStr">
         <is>
           <t>Дмитрий Ковалев</t>
         </is>
       </c>
-      <c r="C11" s="26" t="n">
+      <c r="C11" s="111" t="n">
         <v>5</v>
       </c>
-      <c r="D11" s="64" t="n">
+      <c r="D11" s="117" t="n">
         <v>6.2</v>
       </c>
-      <c r="E11" s="26" t="inlineStr">
+      <c r="E11" s="111" t="inlineStr">
         <is>
           <t>40.0%</t>
         </is>
       </c>
-      <c r="F11" s="26" t="inlineStr">
+      <c r="F11" s="111" t="inlineStr">
         <is>
           <t>72% / 28%</t>
         </is>
       </c>
-      <c r="G11" s="26" t="n">
+      <c r="G11" s="111" t="n">
         <v>3</v>
       </c>
-      <c r="H11" s="62" t="n">
+      <c r="H11" s="114" t="n">
         <v>1100000</v>
       </c>
-      <c r="I11" s="17" t="inlineStr">
+      <c r="I11" s="118" t="inlineStr">
         <is>
           <t>🔴 D (Брак речи)</t>
         </is>
       </c>
-      <c r="J11" s="61" t="inlineStr">
+      <c r="J11" s="27" t="inlineStr">
         <is>
           <t>Срыв контакта, перебивание клиента, демпинг скидок</t>
         </is>
       </c>
-      <c r="K11" s="61" t="n"/>
-      <c r="L11" s="61" t="n"/>
-      <c r="M11" s="61" t="n"/>
-      <c r="N11" s="61" t="n"/>
-      <c r="O11" s="61" t="n"/>
-      <c r="P11" s="61" t="n"/>
-      <c r="Q11" s="61" t="n"/>
-      <c r="R11" s="61" t="n"/>
-      <c r="S11" s="61" t="n"/>
-      <c r="T11" s="61" t="n"/>
-      <c r="U11" s="61" t="n"/>
-      <c r="V11" s="61" t="n"/>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="26" t="n">
+      <c r="A12" s="111" t="n">
         <v>5</v>
       </c>
-      <c r="B12" s="8" t="inlineStr">
+      <c r="B12" s="74" t="inlineStr">
         <is>
           <t>Иван Попов</t>
         </is>
       </c>
-      <c r="C12" s="26" t="n">
+      <c r="C12" s="111" t="n">
         <v>4</v>
       </c>
-      <c r="D12" s="64" t="n">
+      <c r="D12" s="117" t="n">
         <v>5.5</v>
       </c>
-      <c r="E12" s="26" t="inlineStr">
+      <c r="E12" s="111" t="inlineStr">
         <is>
           <t>25.0%</t>
         </is>
       </c>
-      <c r="F12" s="26" t="inlineStr">
+      <c r="F12" s="111" t="inlineStr">
         <is>
           <t>79% / 21%</t>
         </is>
       </c>
-      <c r="G12" s="26" t="n">
+      <c r="G12" s="111" t="n">
         <v>3</v>
       </c>
-      <c r="H12" s="62" t="n">
+      <c r="H12" s="114" t="n">
         <v>1100000</v>
       </c>
-      <c r="I12" s="17" t="inlineStr">
+      <c r="I12" s="118" t="inlineStr">
         <is>
           <t>🔴 D (Брак речи)</t>
         </is>
       </c>
-      <c r="J12" s="61" t="inlineStr">
+      <c r="J12" s="27" t="inlineStr">
         <is>
           <t>Режим 'автоответчика', нет попыток закрытия на встречу</t>
         </is>
       </c>
-      <c r="K12" s="61" t="n"/>
-      <c r="L12" s="61" t="n"/>
-      <c r="M12" s="61" t="n"/>
-      <c r="N12" s="61" t="n"/>
-      <c r="O12" s="61" t="n"/>
-      <c r="P12" s="61" t="n"/>
-      <c r="Q12" s="61" t="n"/>
-      <c r="R12" s="61" t="n"/>
-      <c r="S12" s="61" t="n"/>
-      <c r="T12" s="61" t="n"/>
-      <c r="U12" s="61" t="n"/>
-      <c r="V12" s="61" t="n"/>
     </row>
     <row r="13" ht="24" customHeight="1">
       <c r="A13" s="29" t="inlineStr"/>
-      <c r="B13" s="30" t="inlineStr">
+      <c r="B13" s="119" t="inlineStr">
         <is>
           <t>ИТОГО ПО ОТДЕЛУ ПРОДАЖ:</t>
         </is>
       </c>
-      <c r="C13" s="65">
+      <c r="C13" s="120">
         <f>SUM(C8:C12)</f>
         <v/>
       </c>
-      <c r="D13" s="65" t="inlineStr">
+      <c r="D13" s="120" t="inlineStr">
         <is>
           <t>8.9 / 13</t>
         </is>
       </c>
-      <c r="E13" s="65" t="inlineStr">
+      <c r="E13" s="120" t="inlineStr">
         <is>
           <t>60.0%</t>
         </is>
       </c>
-      <c r="F13" s="65" t="inlineStr">
+      <c r="F13" s="120" t="inlineStr">
         <is>
           <t>61% / 39%</t>
         </is>
       </c>
-      <c r="G13" s="65">
+      <c r="G13" s="120">
         <f>SUM(G8:G12)</f>
         <v/>
       </c>
-      <c r="H13" s="31">
+      <c r="H13" s="121">
         <f>SUM(H8:H12)</f>
         <v/>
       </c>
-      <c r="I13" s="66" t="inlineStr">
+      <c r="I13" s="122" t="inlineStr">
         <is>
           <t>⚠️ РИСК</t>
         </is>
       </c>
-      <c r="J13" s="67" t="inlineStr">
+      <c r="J13" s="123" t="inlineStr">
         <is>
           <t>Требуется экспресс-коучинг по отработке возражений</t>
         </is>
       </c>
-      <c r="K13" s="67" t="n"/>
-      <c r="L13" s="67" t="n"/>
-      <c r="M13" s="67" t="n"/>
-      <c r="N13" s="67" t="n"/>
-      <c r="O13" s="67" t="n"/>
-      <c r="P13" s="67" t="n"/>
-      <c r="Q13" s="67" t="n"/>
-      <c r="R13" s="67" t="n"/>
-      <c r="S13" s="67" t="n"/>
-      <c r="T13" s="67" t="n"/>
-      <c r="U13" s="67" t="n"/>
-      <c r="V13" s="67" t="n"/>
     </row>
     <row r="14" ht="12" customHeight="1"/>
     <row r="15" ht="24" customHeight="1">
-      <c r="A15" s="58" t="inlineStr">
+      <c r="A15" s="110" t="inlineStr">
         <is>
           <t>🔍 ДЕТАЛИЗИРОВАННАЯ МАТРИЦА ОЦЕНКИ ЗВОНКОВ ПО ВСЕМ 13 КРИТЕРИЯМ (0 / 1)</t>
         </is>
       </c>
-      <c r="B15" s="58" t="n"/>
-      <c r="C15" s="58" t="n"/>
-      <c r="D15" s="58" t="n"/>
-      <c r="E15" s="58" t="n"/>
-      <c r="F15" s="58" t="n"/>
-      <c r="G15" s="58" t="n"/>
-      <c r="H15" s="58" t="n"/>
-      <c r="I15" s="58" t="n"/>
-      <c r="J15" s="58" t="n"/>
-      <c r="K15" s="58" t="n"/>
-      <c r="L15" s="58" t="n"/>
-      <c r="M15" s="58" t="n"/>
-      <c r="N15" s="58" t="n"/>
-      <c r="O15" s="58" t="n"/>
-      <c r="P15" s="58" t="n"/>
-      <c r="Q15" s="58" t="n"/>
-      <c r="R15" s="58" t="n"/>
-      <c r="S15" s="58" t="n"/>
-      <c r="T15" s="58" t="n"/>
-      <c r="U15" s="58" t="n"/>
-      <c r="V15" s="58" t="n"/>
     </row>
     <row r="16" ht="32" customHeight="1">
       <c r="A16" s="59" t="inlineStr">
@@ -2738,56 +2702,56 @@
       </c>
     </row>
     <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="44" t="inlineStr">
+      <c r="A17" s="124" t="inlineStr">
         <is>
           <t>C-501</t>
         </is>
       </c>
-      <c r="B17" s="61" t="inlineStr">
+      <c r="B17" s="27" t="inlineStr">
         <is>
           <t>D-101 (ООО Вектор Плюс)</t>
         </is>
       </c>
-      <c r="C17" s="26" t="inlineStr">
+      <c r="C17" s="111" t="inlineStr">
         <is>
           <t>Мельников</t>
         </is>
       </c>
-      <c r="D17" s="68" t="n">
+      <c r="D17" s="125" t="n">
         <v>850000</v>
       </c>
-      <c r="E17" s="26" t="inlineStr">
+      <c r="E17" s="111" t="inlineStr">
         <is>
           <t>05:40</t>
         </is>
       </c>
-      <c r="F17" s="26" t="inlineStr">
+      <c r="F17" s="111" t="inlineStr">
         <is>
           <t>КП отправлено</t>
         </is>
       </c>
-      <c r="G17" s="69" t="n">
-        <v>1</v>
-      </c>
-      <c r="H17" s="69" t="n">
-        <v>1</v>
-      </c>
-      <c r="I17" s="69" t="n">
-        <v>1</v>
-      </c>
-      <c r="J17" s="69" t="n">
-        <v>1</v>
-      </c>
-      <c r="K17" s="69" t="n">
-        <v>1</v>
-      </c>
-      <c r="L17" s="69" t="n">
-        <v>1</v>
-      </c>
-      <c r="M17" s="69" t="n">
-        <v>1</v>
-      </c>
-      <c r="N17" s="69" t="n">
+      <c r="G17" s="126" t="n">
+        <v>1</v>
+      </c>
+      <c r="H17" s="126" t="n">
+        <v>1</v>
+      </c>
+      <c r="I17" s="126" t="n">
+        <v>1</v>
+      </c>
+      <c r="J17" s="126" t="n">
+        <v>1</v>
+      </c>
+      <c r="K17" s="126" t="n">
+        <v>1</v>
+      </c>
+      <c r="L17" s="126" t="n">
+        <v>1</v>
+      </c>
+      <c r="M17" s="126" t="n">
+        <v>1</v>
+      </c>
+      <c r="N17" s="126" t="n">
         <v>1</v>
       </c>
       <c r="O17" s="69" t="n">
@@ -2819,56 +2783,56 @@
       </c>
     </row>
     <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="44" t="inlineStr">
+      <c r="A18" s="124" t="inlineStr">
         <is>
           <t>C-502</t>
         </is>
       </c>
-      <c r="B18" s="61" t="inlineStr">
+      <c r="B18" s="27" t="inlineStr">
         <is>
           <t>D-104 (ООО Вектор Плюс)</t>
         </is>
       </c>
-      <c r="C18" s="26" t="inlineStr">
+      <c r="C18" s="111" t="inlineStr">
         <is>
           <t>Васильева</t>
         </is>
       </c>
-      <c r="D18" s="68" t="n">
+      <c r="D18" s="125" t="n">
         <v>850000</v>
       </c>
-      <c r="E18" s="26" t="inlineStr">
+      <c r="E18" s="111" t="inlineStr">
         <is>
           <t>04:20</t>
         </is>
       </c>
-      <c r="F18" s="26" t="inlineStr">
+      <c r="F18" s="111" t="inlineStr">
         <is>
           <t>Переговоры</t>
         </is>
       </c>
-      <c r="G18" s="69" t="n">
-        <v>1</v>
-      </c>
-      <c r="H18" s="69" t="n">
-        <v>1</v>
-      </c>
-      <c r="I18" s="69" t="n">
-        <v>1</v>
-      </c>
-      <c r="J18" s="69" t="n">
-        <v>1</v>
-      </c>
-      <c r="K18" s="69" t="n">
+      <c r="G18" s="126" t="n">
+        <v>1</v>
+      </c>
+      <c r="H18" s="126" t="n">
+        <v>1</v>
+      </c>
+      <c r="I18" s="126" t="n">
+        <v>1</v>
+      </c>
+      <c r="J18" s="126" t="n">
+        <v>1</v>
+      </c>
+      <c r="K18" s="126" t="n">
         <v>1</v>
       </c>
       <c r="L18" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="M18" s="69" t="n">
-        <v>1</v>
-      </c>
-      <c r="N18" s="69" t="n">
+      <c r="M18" s="126" t="n">
+        <v>1</v>
+      </c>
+      <c r="N18" s="126" t="n">
         <v>1</v>
       </c>
       <c r="O18" s="69" t="n">
@@ -2900,30 +2864,30 @@
       </c>
     </row>
     <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="44" t="inlineStr">
+      <c r="A19" s="124" t="inlineStr">
         <is>
           <t>C-503</t>
         </is>
       </c>
-      <c r="B19" s="61" t="inlineStr">
+      <c r="B19" s="27" t="inlineStr">
         <is>
           <t>D-106 (ООО СнабСервис)</t>
         </is>
       </c>
-      <c r="C19" s="26" t="inlineStr">
+      <c r="C19" s="111" t="inlineStr">
         <is>
           <t>Соколова</t>
         </is>
       </c>
-      <c r="D19" s="68" t="n">
+      <c r="D19" s="125" t="n">
         <v>280000</v>
       </c>
-      <c r="E19" s="26" t="inlineStr">
+      <c r="E19" s="111" t="inlineStr">
         <is>
           <t>03:10</t>
         </is>
       </c>
-      <c r="F19" s="26" t="inlineStr">
+      <c r="F19" s="111" t="inlineStr">
         <is>
           <t>Встреча/Демо</t>
         </is>
@@ -2931,22 +2895,22 @@
       <c r="G19" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="H19" s="69" t="n">
-        <v>1</v>
-      </c>
-      <c r="I19" s="69" t="n">
+      <c r="H19" s="126" t="n">
+        <v>1</v>
+      </c>
+      <c r="I19" s="126" t="n">
         <v>1</v>
       </c>
       <c r="J19" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="K19" s="69" t="n">
+      <c r="K19" s="126" t="n">
         <v>1</v>
       </c>
       <c r="L19" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="M19" s="69" t="n">
+      <c r="M19" s="126" t="n">
         <v>1</v>
       </c>
       <c r="N19" s="70" t="n">
@@ -2981,50 +2945,50 @@
       </c>
     </row>
     <row r="20" ht="22" customHeight="1">
-      <c r="A20" s="44" t="inlineStr">
+      <c r="A20" s="124" t="inlineStr">
         <is>
           <t>C-504</t>
         </is>
       </c>
-      <c r="B20" s="61" t="inlineStr">
+      <c r="B20" s="27" t="inlineStr">
         <is>
           <t>D-107 (ООО ТехноПром)</t>
         </is>
       </c>
-      <c r="C20" s="26" t="inlineStr">
+      <c r="C20" s="111" t="inlineStr">
         <is>
           <t>Соколова</t>
         </is>
       </c>
-      <c r="D20" s="68" t="n">
+      <c r="D20" s="125" t="n">
         <v>150000</v>
       </c>
-      <c r="E20" s="26" t="inlineStr">
+      <c r="E20" s="111" t="inlineStr">
         <is>
           <t>06:15</t>
         </is>
       </c>
-      <c r="F20" s="26" t="inlineStr">
+      <c r="F20" s="111" t="inlineStr">
         <is>
           <t>Квалификация</t>
         </is>
       </c>
-      <c r="G20" s="69" t="n">
-        <v>1</v>
-      </c>
-      <c r="H20" s="69" t="n">
-        <v>1</v>
-      </c>
-      <c r="I20" s="69" t="n">
+      <c r="G20" s="126" t="n">
+        <v>1</v>
+      </c>
+      <c r="H20" s="126" t="n">
+        <v>1</v>
+      </c>
+      <c r="I20" s="126" t="n">
         <v>1</v>
       </c>
       <c r="J20" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="K20" s="69" t="n">
-        <v>1</v>
-      </c>
-      <c r="L20" s="69" t="n">
+      <c r="K20" s="126" t="n">
+        <v>1</v>
+      </c>
+      <c r="L20" s="126" t="n">
         <v>1</v>
       </c>
       <c r="M20" s="70" t="n">
@@ -3062,30 +3026,30 @@
       </c>
     </row>
     <row r="21" ht="22" customHeight="1">
-      <c r="A21" s="44" t="inlineStr">
+      <c r="A21" s="124" t="inlineStr">
         <is>
           <t>C-505</t>
         </is>
       </c>
-      <c r="B21" s="61" t="inlineStr">
+      <c r="B21" s="27" t="inlineStr">
         <is>
           <t>D-109 (ООО ПромКомплект)</t>
         </is>
       </c>
-      <c r="C21" s="26" t="inlineStr">
+      <c r="C21" s="111" t="inlineStr">
         <is>
           <t>Ковалев</t>
         </is>
       </c>
-      <c r="D21" s="68" t="n">
+      <c r="D21" s="125" t="n">
         <v>600000</v>
       </c>
-      <c r="E21" s="26" t="inlineStr">
+      <c r="E21" s="111" t="inlineStr">
         <is>
           <t>03:30</t>
         </is>
       </c>
-      <c r="F21" s="26" t="inlineStr">
+      <c r="F21" s="111" t="inlineStr">
         <is>
           <t>КП отправлено</t>
         </is>
@@ -3143,56 +3107,56 @@
       </c>
     </row>
     <row r="22" ht="22" customHeight="1">
-      <c r="A22" s="44" t="inlineStr">
+      <c r="A22" s="124" t="inlineStr">
         <is>
           <t>C-506</t>
         </is>
       </c>
-      <c r="B22" s="61" t="inlineStr">
+      <c r="B22" s="27" t="inlineStr">
         <is>
           <t>D-111 (ООО Глобал Инвест)</t>
         </is>
       </c>
-      <c r="C22" s="26" t="inlineStr">
+      <c r="C22" s="111" t="inlineStr">
         <is>
           <t>Мельников</t>
         </is>
       </c>
-      <c r="D22" s="68" t="n">
+      <c r="D22" s="125" t="n">
         <v>3000000</v>
       </c>
-      <c r="E22" s="26" t="inlineStr">
+      <c r="E22" s="111" t="inlineStr">
         <is>
           <t>07:15</t>
         </is>
       </c>
-      <c r="F22" s="26" t="inlineStr">
+      <c r="F22" s="111" t="inlineStr">
         <is>
           <t>Финальные условия</t>
         </is>
       </c>
-      <c r="G22" s="69" t="n">
-        <v>1</v>
-      </c>
-      <c r="H22" s="69" t="n">
-        <v>1</v>
-      </c>
-      <c r="I22" s="69" t="n">
-        <v>1</v>
-      </c>
-      <c r="J22" s="69" t="n">
-        <v>1</v>
-      </c>
-      <c r="K22" s="69" t="n">
-        <v>1</v>
-      </c>
-      <c r="L22" s="69" t="n">
-        <v>1</v>
-      </c>
-      <c r="M22" s="69" t="n">
-        <v>1</v>
-      </c>
-      <c r="N22" s="69" t="n">
+      <c r="G22" s="126" t="n">
+        <v>1</v>
+      </c>
+      <c r="H22" s="126" t="n">
+        <v>1</v>
+      </c>
+      <c r="I22" s="126" t="n">
+        <v>1</v>
+      </c>
+      <c r="J22" s="126" t="n">
+        <v>1</v>
+      </c>
+      <c r="K22" s="126" t="n">
+        <v>1</v>
+      </c>
+      <c r="L22" s="126" t="n">
+        <v>1</v>
+      </c>
+      <c r="M22" s="126" t="n">
+        <v>1</v>
+      </c>
+      <c r="N22" s="126" t="n">
         <v>1</v>
       </c>
       <c r="O22" s="69" t="n">
@@ -3224,30 +3188,30 @@
       </c>
     </row>
     <row r="23" ht="22" customHeight="1">
-      <c r="A23" s="44" t="inlineStr">
+      <c r="A23" s="124" t="inlineStr">
         <is>
           <t>C-507</t>
         </is>
       </c>
-      <c r="B23" s="61" t="inlineStr">
+      <c r="B23" s="27" t="inlineStr">
         <is>
           <t>D-114 (ООО АльфаТрейд)</t>
         </is>
       </c>
-      <c r="C23" s="26" t="inlineStr">
+      <c r="C23" s="111" t="inlineStr">
         <is>
           <t>Ковалев</t>
         </is>
       </c>
-      <c r="D23" s="68" t="n">
+      <c r="D23" s="125" t="n">
         <v>500000</v>
       </c>
-      <c r="E23" s="26" t="inlineStr">
+      <c r="E23" s="111" t="inlineStr">
         <is>
           <t>04:45</t>
         </is>
       </c>
-      <c r="F23" s="26" t="inlineStr">
+      <c r="F23" s="111" t="inlineStr">
         <is>
           <t>Дожим договора</t>
         </is>
@@ -3255,10 +3219,10 @@
       <c r="G23" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="H23" s="69" t="n">
-        <v>1</v>
-      </c>
-      <c r="I23" s="69" t="n">
+      <c r="H23" s="126" t="n">
+        <v>1</v>
+      </c>
+      <c r="I23" s="126" t="n">
         <v>1</v>
       </c>
       <c r="J23" s="70" t="n">
@@ -3270,7 +3234,7 @@
       <c r="L23" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="M23" s="69" t="n">
+      <c r="M23" s="126" t="n">
         <v>1</v>
       </c>
       <c r="N23" s="70" t="n">
@@ -3305,30 +3269,30 @@
       </c>
     </row>
     <row r="24" ht="22" customHeight="1">
-      <c r="A24" s="44" t="inlineStr">
+      <c r="A24" s="124" t="inlineStr">
         <is>
           <t>C-508</t>
         </is>
       </c>
-      <c r="B24" s="61" t="inlineStr">
+      <c r="B24" s="27" t="inlineStr">
         <is>
           <t>D-118 (ООО СтройХолдинг)</t>
         </is>
       </c>
-      <c r="C24" s="26" t="inlineStr">
+      <c r="C24" s="111" t="inlineStr">
         <is>
           <t>Попов</t>
         </is>
       </c>
-      <c r="D24" s="68" t="n">
+      <c r="D24" s="125" t="n">
         <v>650000</v>
       </c>
-      <c r="E24" s="26" t="inlineStr">
+      <c r="E24" s="111" t="inlineStr">
         <is>
           <t>02:50</t>
         </is>
       </c>
-      <c r="F24" s="26" t="inlineStr">
+      <c r="F24" s="111" t="inlineStr">
         <is>
           <t>Входящий лид</t>
         </is>
@@ -3339,7 +3303,7 @@
       <c r="H24" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="I24" s="69" t="n">
+      <c r="I24" s="126" t="n">
         <v>1</v>
       </c>
       <c r="J24" s="70" t="n">
@@ -3386,53 +3350,53 @@
       </c>
     </row>
     <row r="25" ht="22" customHeight="1">
-      <c r="A25" s="44" t="inlineStr">
+      <c r="A25" s="124" t="inlineStr">
         <is>
           <t>C-509</t>
         </is>
       </c>
-      <c r="B25" s="61" t="inlineStr">
+      <c r="B25" s="27" t="inlineStr">
         <is>
           <t>D-121 (ООО СпецМаш)</t>
         </is>
       </c>
-      <c r="C25" s="26" t="inlineStr">
+      <c r="C25" s="111" t="inlineStr">
         <is>
           <t>Васильева</t>
         </is>
       </c>
-      <c r="D25" s="68" t="n">
+      <c r="D25" s="125" t="n">
         <v>420000</v>
       </c>
-      <c r="E25" s="26" t="inlineStr">
+      <c r="E25" s="111" t="inlineStr">
         <is>
           <t>05:10</t>
         </is>
       </c>
-      <c r="F25" s="26" t="inlineStr">
+      <c r="F25" s="111" t="inlineStr">
         <is>
           <t>Презентация КП</t>
         </is>
       </c>
-      <c r="G25" s="69" t="n">
-        <v>1</v>
-      </c>
-      <c r="H25" s="69" t="n">
-        <v>1</v>
-      </c>
-      <c r="I25" s="69" t="n">
-        <v>1</v>
-      </c>
-      <c r="J25" s="69" t="n">
-        <v>1</v>
-      </c>
-      <c r="K25" s="69" t="n">
-        <v>1</v>
-      </c>
-      <c r="L25" s="69" t="n">
-        <v>1</v>
-      </c>
-      <c r="M25" s="69" t="n">
+      <c r="G25" s="126" t="n">
+        <v>1</v>
+      </c>
+      <c r="H25" s="126" t="n">
+        <v>1</v>
+      </c>
+      <c r="I25" s="126" t="n">
+        <v>1</v>
+      </c>
+      <c r="J25" s="126" t="n">
+        <v>1</v>
+      </c>
+      <c r="K25" s="126" t="n">
+        <v>1</v>
+      </c>
+      <c r="L25" s="126" t="n">
+        <v>1</v>
+      </c>
+      <c r="M25" s="126" t="n">
         <v>1</v>
       </c>
       <c r="N25" s="70" t="n">
@@ -3467,30 +3431,30 @@
       </c>
     </row>
     <row r="26" ht="22" customHeight="1">
-      <c r="A26" s="44" t="inlineStr">
+      <c r="A26" s="124" t="inlineStr">
         <is>
           <t>C-510</t>
         </is>
       </c>
-      <c r="B26" s="61" t="inlineStr">
+      <c r="B26" s="27" t="inlineStr">
         <is>
           <t>D-125 (ООО МегаТранс)</t>
         </is>
       </c>
-      <c r="C26" s="26" t="inlineStr">
+      <c r="C26" s="111" t="inlineStr">
         <is>
           <t>Попов</t>
         </is>
       </c>
-      <c r="D26" s="68" t="n">
+      <c r="D26" s="125" t="n">
         <v>450000</v>
       </c>
-      <c r="E26" s="26" t="inlineStr">
+      <c r="E26" s="111" t="inlineStr">
         <is>
           <t>03:40</t>
         </is>
       </c>
-      <c r="F26" s="26" t="inlineStr">
+      <c r="F26" s="111" t="inlineStr">
         <is>
           <t>Квалификация</t>
         </is>
@@ -3504,16 +3468,16 @@
       <c r="I26" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="J26" s="69" t="n">
-        <v>1</v>
-      </c>
-      <c r="K26" s="69" t="n">
+      <c r="J26" s="126" t="n">
+        <v>1</v>
+      </c>
+      <c r="K26" s="126" t="n">
         <v>1</v>
       </c>
       <c r="L26" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="M26" s="69" t="n">
+      <c r="M26" s="126" t="n">
         <v>1</v>
       </c>
       <c r="N26" s="70" t="n">
@@ -3548,14 +3512,12 @@
       </c>
     </row>
     <row r="27" ht="24" customHeight="1">
-      <c r="A27" s="30" t="inlineStr">
+      <c r="A27" s="119" t="inlineStr">
         <is>
           <t>ИТОГО ПОТЕРЬ И РИСКОВ ПО ЗВОНКАМ:</t>
         </is>
       </c>
-      <c r="B27" s="30" t="n"/>
-      <c r="C27" s="30" t="n"/>
-      <c r="D27" s="71">
+      <c r="D27" s="127">
         <f>SUM(D17:D26)</f>
         <v/>
       </c>
@@ -3590,87 +3552,51 @@
     </row>
     <row r="28" ht="12" customHeight="1"/>
     <row r="29" ht="24" customHeight="1">
-      <c r="A29" s="58" t="inlineStr">
+      <c r="A29" s="110" t="inlineStr">
         <is>
           <t>🚨 РЕЕСТР ДЕФЕКТОВ РЕЧИ: РАСШИФРОВАННЫЕ ЦИТАТЫ ИЗ РАЗГОВОРОВ И РЕШЕНИЯ РОПа</t>
         </is>
       </c>
-      <c r="B29" s="58" t="n"/>
-      <c r="C29" s="58" t="n"/>
-      <c r="D29" s="58" t="n"/>
-      <c r="E29" s="58" t="n"/>
-      <c r="F29" s="58" t="n"/>
-      <c r="G29" s="58" t="n"/>
-      <c r="H29" s="58" t="n"/>
-      <c r="I29" s="58" t="n"/>
-      <c r="J29" s="58" t="n"/>
-      <c r="K29" s="58" t="n"/>
-      <c r="L29" s="58" t="n"/>
-      <c r="M29" s="58" t="n"/>
-      <c r="N29" s="58" t="n"/>
-      <c r="O29" s="58" t="n"/>
-      <c r="P29" s="58" t="n"/>
-      <c r="Q29" s="58" t="n"/>
-      <c r="R29" s="58" t="n"/>
-      <c r="S29" s="58" t="n"/>
-      <c r="T29" s="58" t="n"/>
-      <c r="U29" s="58" t="n"/>
-      <c r="V29" s="58" t="n"/>
     </row>
     <row r="30" ht="26" customHeight="1">
-      <c r="A30" s="25" t="inlineStr">
+      <c r="A30" s="59" t="inlineStr">
         <is>
           <t>Call ID</t>
         </is>
       </c>
-      <c r="B30" s="25" t="inlineStr">
+      <c r="B30" s="59" t="inlineStr">
         <is>
           <t>Сделка / Контрагент</t>
         </is>
       </c>
-      <c r="C30" s="25" t="inlineStr">
+      <c r="C30" s="59" t="inlineStr">
         <is>
           <t>Менеджер</t>
         </is>
       </c>
-      <c r="D30" s="25" t="inlineStr">
+      <c r="D30" s="59" t="inlineStr">
         <is>
           <t>Сумма в риске</t>
         </is>
       </c>
-      <c r="E30" s="25" t="inlineStr">
+      <c r="E30" s="59" t="inlineStr">
         <is>
           <t>Критический дефект речи</t>
         </is>
       </c>
-      <c r="F30" s="25" t="n"/>
-      <c r="G30" s="25" t="inlineStr">
+      <c r="G30" s="59" t="inlineStr">
         <is>
           <t>💬 Цитата из диалога (Расшифровка Whisper Large V3)</t>
         </is>
       </c>
-      <c r="H30" s="25" t="n"/>
-      <c r="I30" s="25" t="n"/>
-      <c r="J30" s="25" t="n"/>
-      <c r="K30" s="25" t="n"/>
-      <c r="L30" s="25" t="n"/>
-      <c r="M30" s="25" t="n"/>
-      <c r="N30" s="25" t="inlineStr">
+      <c r="N30" s="59" t="inlineStr">
         <is>
           <t>🤖 Решение ИИ и Срочное действие РОПа</t>
         </is>
       </c>
-      <c r="O30" s="25" t="n"/>
-      <c r="P30" s="25" t="n"/>
-      <c r="Q30" s="25" t="n"/>
-      <c r="R30" s="25" t="n"/>
-      <c r="S30" s="25" t="n"/>
-      <c r="T30" s="25" t="n"/>
-      <c r="U30" s="25" t="n"/>
-      <c r="V30" s="25" t="n"/>
     </row>
     <row r="31" ht="60" customHeight="1">
-      <c r="A31" s="44" t="inlineStr">
+      <c r="A31" s="124" t="inlineStr">
         <is>
           <t>C-505</t>
         </is>
@@ -3680,12 +3606,12 @@
           <t>D-109 (ООО «ПромКомплект»)</t>
         </is>
       </c>
-      <c r="C31" s="26" t="inlineStr">
+      <c r="C31" s="111" t="inlineStr">
         <is>
           <t>Дмитрий Ковалев</t>
         </is>
       </c>
-      <c r="D31" s="62" t="n">
+      <c r="D31" s="114" t="n">
         <v>600000</v>
       </c>
       <c r="E31" s="75" t="inlineStr">
@@ -3693,34 +3619,19 @@
           <t>Срыв контакта / грубость при цене</t>
         </is>
       </c>
-      <c r="F31" s="75" t="n"/>
       <c r="G31" s="76" t="inlineStr">
         <is>
           <t>Клиент: «Почему у вас смета на 15% выше рынка?» → Менеджер: «Не знаю, везде всё дорожает. Не устраивает — берите у конкурентов без гарантии»</t>
         </is>
       </c>
-      <c r="H31" s="76" t="n"/>
-      <c r="I31" s="76" t="n"/>
-      <c r="J31" s="76" t="n"/>
-      <c r="K31" s="76" t="n"/>
-      <c r="L31" s="76" t="n"/>
-      <c r="M31" s="76" t="n"/>
       <c r="N31" s="77" t="inlineStr">
         <is>
           <t>🚨 Экстренный звонок РОПа ЛПР до 12:00: принести извинения за консультацию, перехватить сделку, дать проект со спец-гарантией 24 мес.</t>
         </is>
       </c>
-      <c r="O31" s="77" t="n"/>
-      <c r="P31" s="77" t="n"/>
-      <c r="Q31" s="77" t="n"/>
-      <c r="R31" s="77" t="n"/>
-      <c r="S31" s="77" t="n"/>
-      <c r="T31" s="77" t="n"/>
-      <c r="U31" s="77" t="n"/>
-      <c r="V31" s="77" t="n"/>
     </row>
     <row r="32" ht="60" customHeight="1">
-      <c r="A32" s="44" t="inlineStr">
+      <c r="A32" s="124" t="inlineStr">
         <is>
           <t>C-503</t>
         </is>
@@ -3730,12 +3641,12 @@
           <t>D-106 (ООО «СнабСервис»)</t>
         </is>
       </c>
-      <c r="C32" s="26" t="inlineStr">
+      <c r="C32" s="111" t="inlineStr">
         <is>
           <t>Анна Соколова</t>
         </is>
       </c>
-      <c r="D32" s="62" t="n">
+      <c r="D32" s="114" t="n">
         <v>280000</v>
       </c>
       <c r="E32" s="75" t="inlineStr">
@@ -3743,34 +3654,19 @@
           <t>Слив жесткого Next Step (в никуда)</t>
         </is>
       </c>
-      <c r="F32" s="75" t="n"/>
       <c r="G32" s="76" t="inlineStr">
         <is>
           <t>Менеджер: «Я вам КП на почту сбросила, посмотрите когда время будет». Клиент: «Хорошо, если что наберу»</t>
         </is>
       </c>
-      <c r="H32" s="76" t="n"/>
-      <c r="I32" s="76" t="n"/>
-      <c r="J32" s="76" t="n"/>
-      <c r="K32" s="76" t="n"/>
-      <c r="L32" s="76" t="n"/>
-      <c r="M32" s="76" t="n"/>
       <c r="N32" s="77" t="inlineStr">
         <is>
           <t>Направить клиенту в WhatsApp 2 конкретных слота встречи (сегодня 16:00 / завтра 11:30) с демонстрацией интеграции с CRM.</t>
         </is>
       </c>
-      <c r="O32" s="77" t="n"/>
-      <c r="P32" s="77" t="n"/>
-      <c r="Q32" s="77" t="n"/>
-      <c r="R32" s="77" t="n"/>
-      <c r="S32" s="77" t="n"/>
-      <c r="T32" s="77" t="n"/>
-      <c r="U32" s="77" t="n"/>
-      <c r="V32" s="77" t="n"/>
     </row>
     <row r="33" ht="60" customHeight="1">
-      <c r="A33" s="44" t="inlineStr">
+      <c r="A33" s="124" t="inlineStr">
         <is>
           <t>C-507</t>
         </is>
@@ -3780,12 +3676,12 @@
           <t>D-114 (ООО «АльфаТрейд»)</t>
         </is>
       </c>
-      <c r="C33" s="26" t="inlineStr">
+      <c r="C33" s="111" t="inlineStr">
         <is>
           <t>Дмитрий Ковалев</t>
         </is>
       </c>
-      <c r="D33" s="62" t="n">
+      <c r="D33" s="114" t="n">
         <v>500000</v>
       </c>
       <c r="E33" s="75" t="inlineStr">
@@ -3793,34 +3689,19 @@
           <t>Необоснованная скидка вместо ценности</t>
         </is>
       </c>
-      <c r="F33" s="75" t="n"/>
       <c r="G33" s="76" t="inlineStr">
         <is>
           <t>Клиент: «У нас бюджет строго ограничен». Менеджер: «Ну ладно, согласую вам скидку 10% прямо сейчас»</t>
         </is>
       </c>
-      <c r="H33" s="76" t="n"/>
-      <c r="I33" s="76" t="n"/>
-      <c r="J33" s="76" t="n"/>
-      <c r="K33" s="76" t="n"/>
-      <c r="L33" s="76" t="n"/>
-      <c r="M33" s="76" t="n"/>
       <c r="N33" s="77" t="inlineStr">
         <is>
           <t>Заблокировать выставление счета со скидкой в CRM. РОПу пересогласовать условия: скидка 5% только в обмен на 100% предоплату за 24ч.</t>
         </is>
       </c>
-      <c r="O33" s="77" t="n"/>
-      <c r="P33" s="77" t="n"/>
-      <c r="Q33" s="77" t="n"/>
-      <c r="R33" s="77" t="n"/>
-      <c r="S33" s="77" t="n"/>
-      <c r="T33" s="77" t="n"/>
-      <c r="U33" s="77" t="n"/>
-      <c r="V33" s="77" t="n"/>
     </row>
     <row r="34" ht="60" customHeight="1">
-      <c r="A34" s="44" t="inlineStr">
+      <c r="A34" s="124" t="inlineStr">
         <is>
           <t>C-508</t>
         </is>
@@ -3830,12 +3711,12 @@
           <t>D-118 (ООО «СтройХолдинг»)</t>
         </is>
       </c>
-      <c r="C34" s="26" t="inlineStr">
+      <c r="C34" s="111" t="inlineStr">
         <is>
           <t>Иван Попов</t>
         </is>
       </c>
-      <c r="D34" s="62" t="n">
+      <c r="D34" s="114" t="n">
         <v>650000</v>
       </c>
       <c r="E34" s="75" t="inlineStr">
@@ -3843,34 +3724,19 @@
           <t>Слив возражения «Я подумаю»</t>
         </is>
       </c>
-      <c r="F34" s="75" t="n"/>
       <c r="G34" s="76" t="inlineStr">
         <is>
           <t>Клиент: «Нам нужно всё обдумать и посоветоваться с руководством». Менеджер: «Да, конечно, думайте» (повесил трубку)</t>
         </is>
       </c>
-      <c r="H34" s="76" t="n"/>
-      <c r="I34" s="76" t="n"/>
-      <c r="J34" s="76" t="n"/>
-      <c r="K34" s="76" t="n"/>
-      <c r="L34" s="76" t="n"/>
-      <c r="M34" s="76" t="n"/>
       <c r="N34" s="77" t="inlineStr">
         <is>
           <t>Передать лида старшему КАМу. Отправить в WhatsApp отраслевой кейс с аналогичным объектом и окупаемостью за 21 день.</t>
         </is>
       </c>
-      <c r="O34" s="77" t="n"/>
-      <c r="P34" s="77" t="n"/>
-      <c r="Q34" s="77" t="n"/>
-      <c r="R34" s="77" t="n"/>
-      <c r="S34" s="77" t="n"/>
-      <c r="T34" s="77" t="n"/>
-      <c r="U34" s="77" t="n"/>
-      <c r="V34" s="77" t="n"/>
     </row>
     <row r="35" ht="60" customHeight="1">
-      <c r="A35" s="44" t="inlineStr">
+      <c r="A35" s="124" t="inlineStr">
         <is>
           <t>C-510</t>
         </is>
@@ -3880,12 +3746,12 @@
           <t>D-125 (ООО «МегаТранс»)</t>
         </is>
       </c>
-      <c r="C35" s="26" t="inlineStr">
+      <c r="C35" s="111" t="inlineStr">
         <is>
           <t>Иван Попов</t>
         </is>
       </c>
-      <c r="D35" s="62" t="n">
+      <c r="D35" s="114" t="n">
         <v>450000</v>
       </c>
       <c r="E35" s="75" t="inlineStr">
@@ -3893,128 +3759,77 @@
           <t>Режим автоответчика, не выявлен ЛПР</t>
         </is>
       </c>
-      <c r="F35" s="75" t="n"/>
       <c r="G35" s="76" t="inlineStr">
         <is>
           <t>Менеджер 5 минут зачитывал прайс-лист секретарю, не спросив, кто принимает решение по закупкам</t>
         </is>
       </c>
-      <c r="H35" s="76" t="n"/>
-      <c r="I35" s="76" t="n"/>
-      <c r="J35" s="76" t="n"/>
-      <c r="K35" s="76" t="n"/>
-      <c r="L35" s="76" t="n"/>
-      <c r="M35" s="76" t="n"/>
       <c r="N35" s="77" t="inlineStr">
         <is>
           <t>Разбор на летучке: регламент квалификации BANT. Назначить повторный звонок с прямым выходом на генерального директора.</t>
         </is>
       </c>
-      <c r="O35" s="77" t="n"/>
-      <c r="P35" s="77" t="n"/>
-      <c r="Q35" s="77" t="n"/>
-      <c r="R35" s="77" t="n"/>
-      <c r="S35" s="77" t="n"/>
-      <c r="T35" s="77" t="n"/>
-      <c r="U35" s="77" t="n"/>
-      <c r="V35" s="77" t="n"/>
     </row>
     <row r="36" ht="12" customHeight="1"/>
     <row r="37" ht="24" customHeight="1">
-      <c r="A37" s="58" t="inlineStr">
+      <c r="A37" s="110" t="inlineStr">
         <is>
           <t>📋 ЭТАЛОННЫЙ СТАНДАРТ 13 КРИТЕРИЕВ ОЦЕНКИ B2B-ДИАЛОГОВ (WHISPER LARGE V3 + LLM SUPERVISOR)</t>
         </is>
       </c>
-      <c r="B37" s="58" t="n"/>
-      <c r="C37" s="58" t="n"/>
-      <c r="D37" s="58" t="n"/>
-      <c r="E37" s="58" t="n"/>
-      <c r="F37" s="58" t="n"/>
-      <c r="G37" s="58" t="n"/>
-      <c r="H37" s="58" t="n"/>
-      <c r="I37" s="58" t="n"/>
-      <c r="J37" s="58" t="n"/>
-      <c r="K37" s="58" t="n"/>
-      <c r="L37" s="58" t="n"/>
-      <c r="M37" s="58" t="n"/>
-      <c r="N37" s="58" t="n"/>
-      <c r="O37" s="58" t="n"/>
-      <c r="P37" s="58" t="n"/>
-      <c r="Q37" s="58" t="n"/>
-      <c r="R37" s="58" t="n"/>
-      <c r="S37" s="58" t="n"/>
-      <c r="T37" s="58" t="n"/>
-      <c r="U37" s="58" t="n"/>
-      <c r="V37" s="58" t="n"/>
     </row>
     <row r="38" ht="26" customHeight="1">
-      <c r="A38" s="25" t="inlineStr">
+      <c r="A38" s="59" t="inlineStr">
         <is>
           <t>№</t>
         </is>
       </c>
-      <c r="B38" s="25" t="inlineStr">
+      <c r="B38" s="59" t="inlineStr">
         <is>
           <t>Параметр оценки диалога</t>
         </is>
       </c>
-      <c r="C38" s="25" t="inlineStr">
+      <c r="C38" s="59" t="inlineStr">
         <is>
           <t>Вес</t>
         </is>
       </c>
-      <c r="D38" s="25" t="inlineStr">
+      <c r="D38" s="59" t="inlineStr">
         <is>
           <t>Приоритет</t>
         </is>
       </c>
-      <c r="E38" s="25" t="inlineStr">
+      <c r="E38" s="59" t="inlineStr">
         <is>
           <t>Что проверяет алгоритм ИИ (Суть критерия)</t>
         </is>
       </c>
-      <c r="F38" s="25" t="n"/>
-      <c r="G38" s="25" t="n"/>
-      <c r="H38" s="25" t="inlineStr">
+      <c r="H38" s="59" t="inlineStr">
         <is>
           <t>Маркеры дефекта в речи (Почему сделка срывается)</t>
         </is>
       </c>
-      <c r="I38" s="25" t="n"/>
-      <c r="J38" s="25" t="n"/>
-      <c r="K38" s="25" t="n"/>
-      <c r="L38" s="25" t="n"/>
-      <c r="M38" s="25" t="inlineStr">
+      <c r="M38" s="59" t="inlineStr">
         <is>
           <t>Coaching Tip: как обучить менеджера и защитить выручку</t>
         </is>
       </c>
-      <c r="N38" s="25" t="n"/>
-      <c r="O38" s="25" t="n"/>
-      <c r="P38" s="25" t="n"/>
-      <c r="Q38" s="25" t="n"/>
-      <c r="R38" s="25" t="n"/>
-      <c r="S38" s="25" t="n"/>
-      <c r="T38" s="25" t="n"/>
-      <c r="U38" s="25" t="n"/>
-      <c r="V38" s="25" t="n"/>
     </row>
     <row r="39" ht="46" customHeight="1">
-      <c r="A39" s="26" t="n">
-        <v>1</v>
-      </c>
-      <c r="B39" s="8" t="inlineStr">
+      <c r="A39" s="111" t="n">
+        <v>1</v>
+      </c>
+      <c r="B39" s="74" t="inlineStr">
         <is>
           <t>Жёсткий Next Step</t>
         </is>
       </c>
-      <c r="C39" s="26" t="inlineStr">
+      <c r="C39" s="111" t="inlineStr">
         <is>
           <t>2.0x</t>
         </is>
       </c>
-      <c r="D39" s="17" t="inlineStr">
+      <c r="D39" s="118" t="inlineStr">
         <is>
           <t>🔴 P0 (Критический)</t>
         </is>
@@ -4024,47 +3839,32 @@
           <t>Зафиксирована точная дата и время следующего контакта (календарный слот)</t>
         </is>
       </c>
-      <c r="F39" s="27" t="n"/>
-      <c r="G39" s="27" t="n"/>
       <c r="H39" s="78" t="inlineStr">
         <is>
           <t>«Я вам перезвоню на днях», «Подумайте, наберите», отпускание без времени</t>
         </is>
       </c>
-      <c r="I39" s="78" t="n"/>
-      <c r="J39" s="78" t="n"/>
-      <c r="K39" s="78" t="n"/>
-      <c r="L39" s="78" t="n"/>
       <c r="M39" s="74" t="inlineStr">
         <is>
           <t>Внедрить обязательный вопрос в конце диалога: «Во вторник в 14:30 или в среду в 11:00 удобно?»</t>
         </is>
       </c>
-      <c r="N39" s="74" t="n"/>
-      <c r="O39" s="74" t="n"/>
-      <c r="P39" s="74" t="n"/>
-      <c r="Q39" s="74" t="n"/>
-      <c r="R39" s="74" t="n"/>
-      <c r="S39" s="74" t="n"/>
-      <c r="T39" s="74" t="n"/>
-      <c r="U39" s="74" t="n"/>
-      <c r="V39" s="74" t="n"/>
     </row>
     <row r="40" ht="46" customHeight="1">
-      <c r="A40" s="26" t="n">
+      <c r="A40" s="111" t="n">
         <v>2</v>
       </c>
-      <c r="B40" s="8" t="inlineStr">
+      <c r="B40" s="74" t="inlineStr">
         <is>
           <t>Инициатива диалога</t>
         </is>
       </c>
-      <c r="C40" s="26" t="inlineStr">
+      <c r="C40" s="111" t="inlineStr">
         <is>
           <t>1.0x</t>
         </is>
       </c>
-      <c r="D40" s="20" t="inlineStr">
+      <c r="D40" s="116" t="inlineStr">
         <is>
           <t>🟡 P1 (Высокий)</t>
         </is>
@@ -4074,47 +3874,32 @@
           <t>Менеджер ведёт диалог вопросами, держит сценарий, а не работает автоответчиком</t>
         </is>
       </c>
-      <c r="F40" s="27" t="n"/>
-      <c r="G40" s="27" t="n"/>
       <c r="H40" s="78" t="inlineStr">
         <is>
           <t>Клиент задает все вопросы сам, менеджер только отвечает короткими репликами</t>
         </is>
       </c>
-      <c r="I40" s="78" t="n"/>
-      <c r="J40" s="78" t="n"/>
-      <c r="K40" s="78" t="n"/>
-      <c r="L40" s="78" t="n"/>
       <c r="M40" s="74" t="inlineStr">
         <is>
           <t>Правило «Ответ + Встречный вопрос». Завершать каждую реплику квалифицирующим вопросом.</t>
         </is>
       </c>
-      <c r="N40" s="74" t="n"/>
-      <c r="O40" s="74" t="n"/>
-      <c r="P40" s="74" t="n"/>
-      <c r="Q40" s="74" t="n"/>
-      <c r="R40" s="74" t="n"/>
-      <c r="S40" s="74" t="n"/>
-      <c r="T40" s="74" t="n"/>
-      <c r="U40" s="74" t="n"/>
-      <c r="V40" s="74" t="n"/>
     </row>
     <row r="41" ht="46" customHeight="1">
-      <c r="A41" s="26" t="n">
+      <c r="A41" s="111" t="n">
         <v>3</v>
       </c>
-      <c r="B41" s="8" t="inlineStr">
+      <c r="B41" s="74" t="inlineStr">
         <is>
           <t>Квалификация ЛПР / ЛВПР</t>
         </is>
       </c>
-      <c r="C41" s="26" t="inlineStr">
+      <c r="C41" s="111" t="inlineStr">
         <is>
           <t>1.5x</t>
         </is>
       </c>
-      <c r="D41" s="17" t="inlineStr">
+      <c r="D41" s="118" t="inlineStr">
         <is>
           <t>🔴 P0 (Критический)</t>
         </is>
@@ -4124,47 +3909,32 @@
           <t>Установлен статус собеседника: принимает ли решения по бюджету и согласованию</t>
         </is>
       </c>
-      <c r="F41" s="27" t="n"/>
-      <c r="G41" s="27" t="n"/>
       <c r="H41" s="78" t="inlineStr">
         <is>
           <t>Трата 40 минут на презентацию инженеру или секретарю без полномочий подписания</t>
         </is>
       </c>
-      <c r="I41" s="78" t="n"/>
-      <c r="J41" s="78" t="n"/>
-      <c r="K41" s="78" t="n"/>
-      <c r="L41" s="78" t="n"/>
       <c r="M41" s="74" t="inlineStr">
         <is>
           <t>«Кто кроме вас участвует в согласовании проекта и утверждении финансового бюджета?»</t>
         </is>
       </c>
-      <c r="N41" s="74" t="n"/>
-      <c r="O41" s="74" t="n"/>
-      <c r="P41" s="74" t="n"/>
-      <c r="Q41" s="74" t="n"/>
-      <c r="R41" s="74" t="n"/>
-      <c r="S41" s="74" t="n"/>
-      <c r="T41" s="74" t="n"/>
-      <c r="U41" s="74" t="n"/>
-      <c r="V41" s="74" t="n"/>
     </row>
     <row r="42" ht="46" customHeight="1">
-      <c r="A42" s="26" t="n">
+      <c r="A42" s="111" t="n">
         <v>4</v>
       </c>
-      <c r="B42" s="8" t="inlineStr">
+      <c r="B42" s="74" t="inlineStr">
         <is>
           <t>Выявление болей и срочности</t>
         </is>
       </c>
-      <c r="C42" s="26" t="inlineStr">
+      <c r="C42" s="111" t="inlineStr">
         <is>
           <t>1.2x</t>
         </is>
       </c>
-      <c r="D42" s="20" t="inlineStr">
+      <c r="D42" s="116" t="inlineStr">
         <is>
           <t>🟡 P1 (Высокий)</t>
         </is>
@@ -4174,47 +3944,32 @@
           <t>Понятна ли бизнес-задача клиента, текущие потери и дедлайн решения проблемы</t>
         </is>
       </c>
-      <c r="F42" s="27" t="n"/>
-      <c r="G42" s="27" t="n"/>
       <c r="H42" s="78" t="inlineStr">
         <is>
           <t>Менеджер сразу начинает презентовать продукт, не узнав текущую ситуацию клиента</t>
         </is>
       </c>
-      <c r="I42" s="78" t="n"/>
-      <c r="J42" s="78" t="n"/>
-      <c r="K42" s="78" t="n"/>
-      <c r="L42" s="78" t="n"/>
       <c r="M42" s="74" t="inlineStr">
         <is>
           <t>Сначала диагностика по методологии SPIN/BANT, затем презентация под конкретную боль.</t>
         </is>
       </c>
-      <c r="N42" s="74" t="n"/>
-      <c r="O42" s="74" t="n"/>
-      <c r="P42" s="74" t="n"/>
-      <c r="Q42" s="74" t="n"/>
-      <c r="R42" s="74" t="n"/>
-      <c r="S42" s="74" t="n"/>
-      <c r="T42" s="74" t="n"/>
-      <c r="U42" s="74" t="n"/>
-      <c r="V42" s="74" t="n"/>
     </row>
     <row r="43" ht="46" customHeight="1">
-      <c r="A43" s="26" t="n">
+      <c r="A43" s="111" t="n">
         <v>5</v>
       </c>
-      <c r="B43" s="8" t="inlineStr">
+      <c r="B43" s="74" t="inlineStr">
         <is>
           <t>Отработка возражения «Дорого»</t>
         </is>
       </c>
-      <c r="C43" s="26" t="inlineStr">
+      <c r="C43" s="111" t="inlineStr">
         <is>
           <t>1.5x</t>
         </is>
       </c>
-      <c r="D43" s="17" t="inlineStr">
+      <c r="D43" s="118" t="inlineStr">
         <is>
           <t>🔴 P0 (Критический)</t>
         </is>
@@ -4224,47 +3979,32 @@
           <t>Обоснование ценности, расчет ROI/окупаемости, рассрочка (без моментальной скидки)</t>
         </is>
       </c>
-      <c r="F43" s="27" t="n"/>
-      <c r="G43" s="27" t="n"/>
       <c r="H43" s="78" t="inlineStr">
         <is>
           <t>Моментальная скидка при первом сомнении клиента или согласие («Да, у нас недешево»)</t>
         </is>
       </c>
-      <c r="I43" s="78" t="n"/>
-      <c r="J43" s="78" t="n"/>
-      <c r="K43" s="78" t="n"/>
-      <c r="L43" s="78" t="n"/>
       <c r="M43" s="74" t="inlineStr">
         <is>
           <t>Обосновать окупаемость: показать, сколько клиент теряет каждый день без внедрения решения.</t>
         </is>
       </c>
-      <c r="N43" s="74" t="n"/>
-      <c r="O43" s="74" t="n"/>
-      <c r="P43" s="74" t="n"/>
-      <c r="Q43" s="74" t="n"/>
-      <c r="R43" s="74" t="n"/>
-      <c r="S43" s="74" t="n"/>
-      <c r="T43" s="74" t="n"/>
-      <c r="U43" s="74" t="n"/>
-      <c r="V43" s="74" t="n"/>
     </row>
     <row r="44" ht="46" customHeight="1">
-      <c r="A44" s="26" t="n">
+      <c r="A44" s="111" t="n">
         <v>6</v>
       </c>
-      <c r="B44" s="8" t="inlineStr">
+      <c r="B44" s="74" t="inlineStr">
         <is>
           <t>Отработка «Я подумаю»</t>
         </is>
       </c>
-      <c r="C44" s="26" t="inlineStr">
+      <c r="C44" s="111" t="inlineStr">
         <is>
           <t>1.0x</t>
         </is>
       </c>
-      <c r="D44" s="20" t="inlineStr">
+      <c r="D44" s="116" t="inlineStr">
         <is>
           <t>🟡 P1 (Высокий)</t>
         </is>
@@ -4274,47 +4014,32 @@
           <t>Вскрытие истинного сомнения клиента, а не молчаливое отпускание в архив</t>
         </is>
       </c>
-      <c r="F44" s="27" t="n"/>
-      <c r="G44" s="27" t="n"/>
       <c r="H44" s="78" t="inlineStr">
         <is>
           <t>«Хорошо, думайте, ждем вашего звонка», завершение диалога на неопределенности</t>
         </is>
       </c>
-      <c r="I44" s="78" t="n"/>
-      <c r="J44" s="78" t="n"/>
-      <c r="K44" s="78" t="n"/>
-      <c r="L44" s="78" t="n"/>
       <c r="M44" s="74" t="inlineStr">
         <is>
           <t>«Алексей, обычно говорят 'подумаю', когда смущает цена или функционал. Что именно из этого?»</t>
         </is>
       </c>
-      <c r="N44" s="74" t="n"/>
-      <c r="O44" s="74" t="n"/>
-      <c r="P44" s="74" t="n"/>
-      <c r="Q44" s="74" t="n"/>
-      <c r="R44" s="74" t="n"/>
-      <c r="S44" s="74" t="n"/>
-      <c r="T44" s="74" t="n"/>
-      <c r="U44" s="74" t="n"/>
-      <c r="V44" s="74" t="n"/>
     </row>
     <row r="45" ht="46" customHeight="1">
-      <c r="A45" s="26" t="n">
+      <c r="A45" s="111" t="n">
         <v>7</v>
       </c>
-      <c r="B45" s="8" t="inlineStr">
+      <c r="B45" s="74" t="inlineStr">
         <is>
           <t>Презентация через кейсы и цифры</t>
         </is>
       </c>
-      <c r="C45" s="26" t="inlineStr">
+      <c r="C45" s="111" t="inlineStr">
         <is>
           <t>1.0x</t>
         </is>
       </c>
-      <c r="D45" s="20" t="inlineStr">
+      <c r="D45" s="116" t="inlineStr">
         <is>
           <t>🟡 P1 (Высокий)</t>
         </is>
@@ -4324,47 +4049,32 @@
           <t>Приведение аналогичных проектов, оцифрованных результатов и сроков возврата</t>
         </is>
       </c>
-      <c r="F45" s="27" t="n"/>
-      <c r="G45" s="27" t="n"/>
       <c r="H45" s="78" t="inlineStr">
         <is>
           <t>Абстрактные слова «мы надежные», «у нас высокое качество» без конкретных фактов</t>
         </is>
       </c>
-      <c r="I45" s="78" t="n"/>
-      <c r="J45" s="78" t="n"/>
-      <c r="K45" s="78" t="n"/>
-      <c r="L45" s="78" t="n"/>
       <c r="M45" s="74" t="inlineStr">
         <is>
           <t>Показать схожий кейс из отрасли клиента: «Для завода X мы сократили потери на 1.4 млн ₽ за 21 день».</t>
         </is>
       </c>
-      <c r="N45" s="74" t="n"/>
-      <c r="O45" s="74" t="n"/>
-      <c r="P45" s="74" t="n"/>
-      <c r="Q45" s="74" t="n"/>
-      <c r="R45" s="74" t="n"/>
-      <c r="S45" s="74" t="n"/>
-      <c r="T45" s="74" t="n"/>
-      <c r="U45" s="74" t="n"/>
-      <c r="V45" s="74" t="n"/>
     </row>
     <row r="46" ht="46" customHeight="1">
-      <c r="A46" s="26" t="n">
+      <c r="A46" s="111" t="n">
         <v>8</v>
       </c>
-      <c r="B46" s="8" t="inlineStr">
+      <c r="B46" s="74" t="inlineStr">
         <is>
           <t>Попытка закрытия сделки</t>
         </is>
       </c>
-      <c r="C46" s="26" t="inlineStr">
+      <c r="C46" s="111" t="inlineStr">
         <is>
           <t>1.5x</t>
         </is>
       </c>
-      <c r="D46" s="17" t="inlineStr">
+      <c r="D46" s="118" t="inlineStr">
         <is>
           <t>🔴 P0 (Критический)</t>
         </is>
@@ -4374,47 +4084,32 @@
           <t>Прямое предложение заключить договор, забронировать слот аудита или выставить счет</t>
         </is>
       </c>
-      <c r="F46" s="27" t="n"/>
-      <c r="G46" s="27" t="n"/>
       <c r="H46" s="78" t="inlineStr">
         <is>
           <t>Разговор закончился тепло, но менеджер не предложил сделать следующий шаг к оплате</t>
         </is>
       </c>
-      <c r="I46" s="78" t="n"/>
-      <c r="J46" s="78" t="n"/>
-      <c r="K46" s="78" t="n"/>
-      <c r="L46" s="78" t="n"/>
       <c r="M46" s="74" t="inlineStr">
         <is>
           <t>«Если все параметры подходят, предлагаю сегодня запустить пилот. Куда отправить договор?»</t>
         </is>
       </c>
-      <c r="N46" s="74" t="n"/>
-      <c r="O46" s="74" t="n"/>
-      <c r="P46" s="74" t="n"/>
-      <c r="Q46" s="74" t="n"/>
-      <c r="R46" s="74" t="n"/>
-      <c r="S46" s="74" t="n"/>
-      <c r="T46" s="74" t="n"/>
-      <c r="U46" s="74" t="n"/>
-      <c r="V46" s="74" t="n"/>
     </row>
     <row r="47" ht="46" customHeight="1">
-      <c r="A47" s="26" t="n">
+      <c r="A47" s="111" t="n">
         <v>9</v>
       </c>
-      <c r="B47" s="8" t="inlineStr">
+      <c r="B47" s="74" t="inlineStr">
         <is>
           <t>Регламент приветствия и повестка</t>
         </is>
       </c>
-      <c r="C47" s="26" t="inlineStr">
+      <c r="C47" s="111" t="inlineStr">
         <is>
           <t>0.8x</t>
         </is>
       </c>
-      <c r="D47" s="79" t="inlineStr">
+      <c r="D47" s="128" t="inlineStr">
         <is>
           <t>🟢 P2 (Стандарт)</t>
         </is>
@@ -4424,47 +4119,32 @@
           <t>Представление имени, компании, уточнение времени и согласование цели разговора</t>
         </is>
       </c>
-      <c r="F47" s="27" t="n"/>
-      <c r="G47" s="27" t="n"/>
       <c r="H47" s="78" t="inlineStr">
         <is>
           <t>Невнятное приветствие, вопрос «Вам удобно говорить?» без обозначения повестки</t>
         </is>
       </c>
-      <c r="I47" s="78" t="n"/>
-      <c r="J47" s="78" t="n"/>
-      <c r="K47" s="78" t="n"/>
-      <c r="L47" s="78" t="n"/>
       <c r="M47" s="74" t="inlineStr">
         <is>
           <t>«Добрый день! Дмитрий, компания RevOps. Звоню по вашей заявке на аудит воронки. Уделите 5 минут?»</t>
         </is>
       </c>
-      <c r="N47" s="74" t="n"/>
-      <c r="O47" s="74" t="n"/>
-      <c r="P47" s="74" t="n"/>
-      <c r="Q47" s="74" t="n"/>
-      <c r="R47" s="74" t="n"/>
-      <c r="S47" s="74" t="n"/>
-      <c r="T47" s="74" t="n"/>
-      <c r="U47" s="74" t="n"/>
-      <c r="V47" s="74" t="n"/>
     </row>
     <row r="48" ht="46" customHeight="1">
-      <c r="A48" s="26" t="n">
+      <c r="A48" s="111" t="n">
         <v>10</v>
       </c>
-      <c r="B48" s="8" t="inlineStr">
+      <c r="B48" s="74" t="inlineStr">
         <is>
           <t>Чистота речи и уверенность</t>
         </is>
       </c>
-      <c r="C48" s="26" t="inlineStr">
+      <c r="C48" s="111" t="inlineStr">
         <is>
           <t>0.8x</t>
         </is>
       </c>
-      <c r="D48" s="79" t="inlineStr">
+      <c r="D48" s="128" t="inlineStr">
         <is>
           <t>🟢 P2 (Стандарт)</t>
         </is>
@@ -4474,47 +4154,32 @@
           <t>Отсутствие слов-паразитов («как бы», «э-э-э»), пауз и извиняющихся интонаций при цене</t>
         </is>
       </c>
-      <c r="F48" s="27" t="n"/>
-      <c r="G48" s="27" t="n"/>
       <c r="H48" s="78" t="inlineStr">
         <is>
           <t>Дрожащий голос при озвучивании чека, слова сомнения («может быть», «наверное»)</t>
         </is>
       </c>
-      <c r="I48" s="78" t="n"/>
-      <c r="J48" s="78" t="n"/>
-      <c r="K48" s="78" t="n"/>
-      <c r="L48" s="78" t="n"/>
       <c r="M48" s="74" t="inlineStr">
         <is>
           <t>Отработать блок цены на тренажере: уверенная пауза после озвучивания стоимости.</t>
         </is>
       </c>
-      <c r="N48" s="74" t="n"/>
-      <c r="O48" s="74" t="n"/>
-      <c r="P48" s="74" t="n"/>
-      <c r="Q48" s="74" t="n"/>
-      <c r="R48" s="74" t="n"/>
-      <c r="S48" s="74" t="n"/>
-      <c r="T48" s="74" t="n"/>
-      <c r="U48" s="74" t="n"/>
-      <c r="V48" s="74" t="n"/>
     </row>
     <row r="49" ht="46" customHeight="1">
-      <c r="A49" s="26" t="n">
+      <c r="A49" s="111" t="n">
         <v>11</v>
       </c>
-      <c r="B49" s="8" t="inlineStr">
+      <c r="B49" s="74" t="inlineStr">
         <is>
           <t>Слушание клиента (Talk/Listen)</t>
         </is>
       </c>
-      <c r="C49" s="26" t="inlineStr">
+      <c r="C49" s="111" t="inlineStr">
         <is>
           <t>1.2x</t>
         </is>
       </c>
-      <c r="D49" s="20" t="inlineStr">
+      <c r="D49" s="116" t="inlineStr">
         <is>
           <t>🟡 P1 (Высокий)</t>
         </is>
@@ -4524,47 +4189,32 @@
           <t>Менеджер слушает клиента не менее 45–50% общего времени разговора</t>
         </is>
       </c>
-      <c r="F49" s="27" t="n"/>
-      <c r="G49" s="27" t="n"/>
       <c r="H49" s="78" t="inlineStr">
         <is>
           <t>Монолог менеджера &gt; 70% времени: клиент молчит и теряет фокус внимания</t>
         </is>
       </c>
-      <c r="I49" s="78" t="n"/>
-      <c r="J49" s="78" t="n"/>
-      <c r="K49" s="78" t="n"/>
-      <c r="L49" s="78" t="n"/>
       <c r="M49" s="74" t="inlineStr">
         <is>
           <t>Держать баланс 50/50. Задавать открытые вопросы и давать клиенту выговориться о проблеме.</t>
         </is>
       </c>
-      <c r="N49" s="74" t="n"/>
-      <c r="O49" s="74" t="n"/>
-      <c r="P49" s="74" t="n"/>
-      <c r="Q49" s="74" t="n"/>
-      <c r="R49" s="74" t="n"/>
-      <c r="S49" s="74" t="n"/>
-      <c r="T49" s="74" t="n"/>
-      <c r="U49" s="74" t="n"/>
-      <c r="V49" s="74" t="n"/>
     </row>
     <row r="50" ht="46" customHeight="1">
-      <c r="A50" s="26" t="n">
+      <c r="A50" s="111" t="n">
         <v>12</v>
       </c>
-      <c r="B50" s="8" t="inlineStr">
+      <c r="B50" s="74" t="inlineStr">
         <is>
           <t>Фиксация договорённостей</t>
         </is>
       </c>
-      <c r="C50" s="26" t="inlineStr">
+      <c r="C50" s="111" t="inlineStr">
         <is>
           <t>1.0x</t>
         </is>
       </c>
-      <c r="D50" s="79" t="inlineStr">
+      <c r="D50" s="128" t="inlineStr">
         <is>
           <t>🟢 P2 (Стандарт)</t>
         </is>
@@ -4574,47 +4224,32 @@
           <t>Резюмирование договоренностей перед окончанием звонка: кто, что и когда делает</t>
         </is>
       </c>
-      <c r="F50" s="27" t="n"/>
-      <c r="G50" s="27" t="n"/>
       <c r="H50" s="78" t="inlineStr">
         <is>
           <t>Диалог оборвался, у клиента и менеджера разное понимание следующих действий</t>
         </is>
       </c>
-      <c r="I50" s="78" t="n"/>
-      <c r="J50" s="78" t="n"/>
-      <c r="K50" s="78" t="n"/>
-      <c r="L50" s="78" t="n"/>
       <c r="M50" s="74" t="inlineStr">
         <is>
           <t>«Итак, резюмирую: я отправляю КП в WhatsApp до 15:00, а завтра в 11:00 мы созваниваемся по условиям».</t>
         </is>
       </c>
-      <c r="N50" s="74" t="n"/>
-      <c r="O50" s="74" t="n"/>
-      <c r="P50" s="74" t="n"/>
-      <c r="Q50" s="74" t="n"/>
-      <c r="R50" s="74" t="n"/>
-      <c r="S50" s="74" t="n"/>
-      <c r="T50" s="74" t="n"/>
-      <c r="U50" s="74" t="n"/>
-      <c r="V50" s="74" t="n"/>
     </row>
     <row r="51" ht="46" customHeight="1">
-      <c r="A51" s="26" t="n">
+      <c r="A51" s="111" t="n">
         <v>13</v>
       </c>
-      <c r="B51" s="8" t="inlineStr">
+      <c r="B51" s="74" t="inlineStr">
         <is>
           <t>Защита маржинальности</t>
         </is>
       </c>
-      <c r="C51" s="26" t="inlineStr">
+      <c r="C51" s="111" t="inlineStr">
         <is>
           <t>1.5x</t>
         </is>
       </c>
-      <c r="D51" s="17" t="inlineStr">
+      <c r="D51" s="118" t="inlineStr">
         <is>
           <t>🔴 P0 (Критический)</t>
         </is>
@@ -4624,421 +4259,137 @@
           <t>Отсутствие необоснованных скидок без встречных уступок по объему или предоплате</t>
         </is>
       </c>
-      <c r="F51" s="27" t="n"/>
-      <c r="G51" s="27" t="n"/>
       <c r="H51" s="78" t="inlineStr">
         <is>
           <t>Раздача скидок из маржи компании без требования 100% предоплаты или большего объема</t>
         </is>
       </c>
-      <c r="I51" s="78" t="n"/>
-      <c r="J51" s="78" t="n"/>
-      <c r="K51" s="78" t="n"/>
-      <c r="L51" s="78" t="n"/>
       <c r="M51" s="74" t="inlineStr">
         <is>
           <t>Скидка возможна только в обмен на ценность: «Готовы дать 5% при оплате счета в течение 24 часов».</t>
         </is>
       </c>
-      <c r="N51" s="74" t="n"/>
-      <c r="O51" s="74" t="n"/>
-      <c r="P51" s="74" t="n"/>
-      <c r="Q51" s="74" t="n"/>
-      <c r="R51" s="74" t="n"/>
-      <c r="S51" s="74" t="n"/>
-      <c r="T51" s="74" t="n"/>
-      <c r="U51" s="74" t="n"/>
-      <c r="V51" s="74" t="n"/>
     </row>
     <row r="52" ht="12" customHeight="1"/>
     <row r="53" ht="24" customHeight="1">
-      <c r="A53" s="58" t="inlineStr">
+      <c r="A53" s="110" t="inlineStr">
         <is>
           <t>💰 ЭКОНОМИЧЕСКИЙ ЭФФЕКТ РЕЧЕВОЙ АНАЛИТИКИ (ROI ВНЕДРЕНИЯ И ОКУПАЕМОСТЬ)</t>
         </is>
       </c>
-      <c r="B53" s="58" t="n"/>
-      <c r="C53" s="58" t="n"/>
-      <c r="D53" s="58" t="n"/>
-      <c r="E53" s="58" t="n"/>
-      <c r="F53" s="58" t="n"/>
-      <c r="G53" s="58" t="n"/>
-      <c r="H53" s="58" t="n"/>
-      <c r="I53" s="58" t="n"/>
-      <c r="J53" s="58" t="n"/>
-      <c r="K53" s="58" t="n"/>
-      <c r="L53" s="58" t="n"/>
-      <c r="M53" s="58" t="n"/>
-      <c r="N53" s="58" t="n"/>
-      <c r="O53" s="58" t="n"/>
-      <c r="P53" s="58" t="n"/>
-      <c r="Q53" s="58" t="n"/>
-      <c r="R53" s="58" t="n"/>
-      <c r="S53" s="58" t="n"/>
-      <c r="T53" s="58" t="n"/>
-      <c r="U53" s="58" t="n"/>
-      <c r="V53" s="58" t="n"/>
     </row>
     <row r="54" ht="26" customHeight="1">
-      <c r="A54" s="25" t="inlineStr">
+      <c r="A54" s="59" t="inlineStr">
         <is>
           <t>Параметр эффекта речевой аналитики</t>
         </is>
       </c>
-      <c r="B54" s="25" t="n"/>
-      <c r="C54" s="25" t="n"/>
-      <c r="D54" s="25" t="inlineStr">
+      <c r="D54" s="59" t="inlineStr">
         <is>
           <t>Значение</t>
         </is>
       </c>
-      <c r="E54" s="25" t="n"/>
-      <c r="F54" s="25" t="inlineStr">
+      <c r="F54" s="59" t="inlineStr">
         <is>
           <t>Комментарий и логика окупаемости</t>
         </is>
       </c>
-      <c r="G54" s="25" t="n"/>
-      <c r="H54" s="25" t="n"/>
-      <c r="I54" s="25" t="n"/>
-      <c r="J54" s="25" t="n"/>
-      <c r="K54" s="25" t="n"/>
-      <c r="L54" s="25" t="n"/>
-      <c r="M54" s="25" t="n"/>
-      <c r="N54" s="25" t="n"/>
-      <c r="O54" s="25" t="n"/>
-      <c r="P54" s="25" t="n"/>
-      <c r="Q54" s="25" t="n"/>
-      <c r="R54" s="25" t="n"/>
-      <c r="S54" s="25" t="n"/>
-      <c r="T54" s="25" t="n"/>
-      <c r="U54" s="25" t="n"/>
-      <c r="V54" s="25" t="n"/>
     </row>
     <row r="55" ht="24" customHeight="1">
-      <c r="A55" s="80" t="inlineStr">
+      <c r="A55" s="74" t="inlineStr">
         <is>
           <t>Текущие потери от брака звонков в месяц (As-Is)</t>
         </is>
       </c>
-      <c r="B55" s="80" t="n"/>
-      <c r="C55" s="80" t="n"/>
-      <c r="D55" s="81" t="n">
+      <c r="D55" s="129" t="n">
         <v>1382500</v>
       </c>
-      <c r="E55" s="81" t="n"/>
-      <c r="F55" s="61" t="inlineStr">
+      <c r="F55" s="27" t="inlineStr">
         <is>
           <t>Сливы на этапе первичного звонка из-за отсутствия Next Step и слабой отработки возражений</t>
         </is>
       </c>
-      <c r="G55" s="61" t="n"/>
-      <c r="H55" s="61" t="n"/>
-      <c r="I55" s="61" t="n"/>
-      <c r="J55" s="61" t="n"/>
-      <c r="K55" s="61" t="n"/>
-      <c r="L55" s="61" t="n"/>
-      <c r="M55" s="61" t="n"/>
-      <c r="N55" s="61" t="n"/>
-      <c r="O55" s="61" t="n"/>
-      <c r="P55" s="61" t="n"/>
-      <c r="Q55" s="61" t="n"/>
-      <c r="R55" s="61" t="n"/>
-      <c r="S55" s="61" t="n"/>
-      <c r="T55" s="61" t="n"/>
-      <c r="U55" s="61" t="n"/>
-      <c r="V55" s="61" t="n"/>
     </row>
     <row r="56" ht="24" customHeight="1">
-      <c r="A56" s="80" t="inlineStr">
+      <c r="A56" s="74" t="inlineStr">
         <is>
           <t>Ожидаемый возврат выручки в кассу (M1 To-Be)</t>
         </is>
       </c>
-      <c r="B56" s="80" t="n"/>
-      <c r="C56" s="80" t="n"/>
-      <c r="D56" s="82" t="n">
+      <c r="D56" s="130" t="n">
         <v>414750</v>
       </c>
-      <c r="E56" s="82" t="n"/>
-      <c r="F56" s="61" t="inlineStr">
+      <c r="F56" s="27" t="inlineStr">
         <is>
           <t>Консервативный сценарий: устранение всего 30% выявленных дефектов речи</t>
         </is>
       </c>
-      <c r="G56" s="61" t="n"/>
-      <c r="H56" s="61" t="n"/>
-      <c r="I56" s="61" t="n"/>
-      <c r="J56" s="61" t="n"/>
-      <c r="K56" s="61" t="n"/>
-      <c r="L56" s="61" t="n"/>
-      <c r="M56" s="61" t="n"/>
-      <c r="N56" s="61" t="n"/>
-      <c r="O56" s="61" t="n"/>
-      <c r="P56" s="61" t="n"/>
-      <c r="Q56" s="61" t="n"/>
-      <c r="R56" s="61" t="n"/>
-      <c r="S56" s="61" t="n"/>
-      <c r="T56" s="61" t="n"/>
-      <c r="U56" s="61" t="n"/>
-      <c r="V56" s="61" t="n"/>
     </row>
     <row r="57" ht="24" customHeight="1">
-      <c r="A57" s="80" t="inlineStr">
+      <c r="A57" s="74" t="inlineStr">
         <is>
           <t>Стоимость модуля речевого ИИ-супервайзера</t>
         </is>
       </c>
-      <c r="B57" s="80" t="n"/>
-      <c r="C57" s="80" t="n"/>
-      <c r="D57" s="83" t="n">
+      <c r="D57" s="131" t="n">
         <v>150000</v>
       </c>
-      <c r="E57" s="83" t="n"/>
-      <c r="F57" s="61" t="inlineStr">
+      <c r="F57" s="27" t="inlineStr">
         <is>
           <t>В составе комплексного 4-недельного спринта оптимизации отдела продаж</t>
         </is>
       </c>
-      <c r="G57" s="61" t="n"/>
-      <c r="H57" s="61" t="n"/>
-      <c r="I57" s="61" t="n"/>
-      <c r="J57" s="61" t="n"/>
-      <c r="K57" s="61" t="n"/>
-      <c r="L57" s="61" t="n"/>
-      <c r="M57" s="61" t="n"/>
-      <c r="N57" s="61" t="n"/>
-      <c r="O57" s="61" t="n"/>
-      <c r="P57" s="61" t="n"/>
-      <c r="Q57" s="61" t="n"/>
-      <c r="R57" s="61" t="n"/>
-      <c r="S57" s="61" t="n"/>
-      <c r="T57" s="61" t="n"/>
-      <c r="U57" s="61" t="n"/>
-      <c r="V57" s="61" t="n"/>
     </row>
     <row r="58" ht="24" customHeight="1">
-      <c r="A58" s="80" t="inlineStr">
+      <c r="A58" s="74" t="inlineStr">
         <is>
           <t>Чистая прибыль компании от внедрения в первый месяц</t>
         </is>
       </c>
-      <c r="B58" s="80" t="n"/>
-      <c r="C58" s="80" t="n"/>
-      <c r="D58" s="82" t="n">
+      <c r="D58" s="130" t="n">
         <v>264750</v>
       </c>
-      <c r="E58" s="82" t="n"/>
-      <c r="F58" s="61" t="inlineStr">
+      <c r="F58" s="27" t="inlineStr">
         <is>
           <t>Чистый денежный плюс в кассе компании уже в первый месяц работы</t>
         </is>
       </c>
-      <c r="G58" s="61" t="n"/>
-      <c r="H58" s="61" t="n"/>
-      <c r="I58" s="61" t="n"/>
-      <c r="J58" s="61" t="n"/>
-      <c r="K58" s="61" t="n"/>
-      <c r="L58" s="61" t="n"/>
-      <c r="M58" s="61" t="n"/>
-      <c r="N58" s="61" t="n"/>
-      <c r="O58" s="61" t="n"/>
-      <c r="P58" s="61" t="n"/>
-      <c r="Q58" s="61" t="n"/>
-      <c r="R58" s="61" t="n"/>
-      <c r="S58" s="61" t="n"/>
-      <c r="T58" s="61" t="n"/>
-      <c r="U58" s="61" t="n"/>
-      <c r="V58" s="61" t="n"/>
     </row>
     <row r="59" ht="24" customHeight="1">
-      <c r="A59" s="80" t="inlineStr">
+      <c r="A59" s="74" t="inlineStr">
         <is>
           <t>Чистый ROI речевой аналитики</t>
         </is>
       </c>
-      <c r="B59" s="80" t="n"/>
-      <c r="C59" s="80" t="n"/>
-      <c r="D59" s="60" t="inlineStr">
+      <c r="D59" s="112" t="inlineStr">
         <is>
           <t>276%</t>
         </is>
       </c>
-      <c r="E59" s="60" t="n"/>
-      <c r="F59" s="61" t="inlineStr">
+      <c r="F59" s="27" t="inlineStr">
         <is>
           <t>Отдача на каждый вложенный рубль в первый месяц</t>
         </is>
       </c>
-      <c r="G59" s="61" t="n"/>
-      <c r="H59" s="61" t="n"/>
-      <c r="I59" s="61" t="n"/>
-      <c r="J59" s="61" t="n"/>
-      <c r="K59" s="61" t="n"/>
-      <c r="L59" s="61" t="n"/>
-      <c r="M59" s="61" t="n"/>
-      <c r="N59" s="61" t="n"/>
-      <c r="O59" s="61" t="n"/>
-      <c r="P59" s="61" t="n"/>
-      <c r="Q59" s="61" t="n"/>
-      <c r="R59" s="61" t="n"/>
-      <c r="S59" s="61" t="n"/>
-      <c r="T59" s="61" t="n"/>
-      <c r="U59" s="61" t="n"/>
-      <c r="V59" s="61" t="n"/>
     </row>
     <row r="60" ht="24" customHeight="1">
-      <c r="A60" s="80" t="inlineStr">
+      <c r="A60" s="74" t="inlineStr">
         <is>
           <t>Срок полной окупаемости модуля</t>
         </is>
       </c>
-      <c r="B60" s="80" t="n"/>
-      <c r="C60" s="80" t="n"/>
-      <c r="D60" s="60" t="inlineStr">
+      <c r="D60" s="112" t="inlineStr">
         <is>
           <t>11 дней</t>
         </is>
       </c>
-      <c r="E60" s="60" t="n"/>
-      <c r="F60" s="61" t="inlineStr">
+      <c r="F60" s="27" t="inlineStr">
         <is>
           <t>Количество рабочих дней до полной окупаемости внедрения речевого ИИ</t>
         </is>
       </c>
-      <c r="G60" s="61" t="n"/>
-      <c r="H60" s="61" t="n"/>
-      <c r="I60" s="61" t="n"/>
-      <c r="J60" s="61" t="n"/>
-      <c r="K60" s="61" t="n"/>
-      <c r="L60" s="61" t="n"/>
-      <c r="M60" s="61" t="n"/>
-      <c r="N60" s="61" t="n"/>
-      <c r="O60" s="61" t="n"/>
-      <c r="P60" s="61" t="n"/>
-      <c r="Q60" s="61" t="n"/>
-      <c r="R60" s="61" t="n"/>
-      <c r="S60" s="61" t="n"/>
-      <c r="T60" s="61" t="n"/>
-      <c r="U60" s="61" t="n"/>
-      <c r="V60" s="61" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="113">
-    <mergeCell ref="D2:F2"/>
-    <mergeCell ref="D60:E60"/>
-    <mergeCell ref="N2:P2"/>
-    <mergeCell ref="M41:V41"/>
-    <mergeCell ref="H43:L43"/>
-    <mergeCell ref="E40:G40"/>
-    <mergeCell ref="H41:L41"/>
-    <mergeCell ref="A29:V29"/>
-    <mergeCell ref="A57:C57"/>
-    <mergeCell ref="H49:L49"/>
-    <mergeCell ref="N31:V31"/>
-    <mergeCell ref="J3:L3"/>
-    <mergeCell ref="A15:V15"/>
-    <mergeCell ref="E34:F34"/>
-    <mergeCell ref="M39:V39"/>
-    <mergeCell ref="J9:V9"/>
-    <mergeCell ref="M48:V48"/>
-    <mergeCell ref="D56:E56"/>
-    <mergeCell ref="N35:V35"/>
-    <mergeCell ref="E42:G42"/>
-    <mergeCell ref="H48:L48"/>
-    <mergeCell ref="E44:G44"/>
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="G33:M33"/>
-    <mergeCell ref="E3:F3"/>
-    <mergeCell ref="H38:L38"/>
-    <mergeCell ref="G35:M35"/>
-    <mergeCell ref="H44:L44"/>
-    <mergeCell ref="A55:C55"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="M38:V38"/>
-    <mergeCell ref="H40:L40"/>
-    <mergeCell ref="E4:F4"/>
-    <mergeCell ref="E46:G46"/>
-    <mergeCell ref="H51:L51"/>
-    <mergeCell ref="F59:V59"/>
-    <mergeCell ref="M43:V43"/>
-    <mergeCell ref="J8:V8"/>
-    <mergeCell ref="F55:V55"/>
-    <mergeCell ref="G4:I4"/>
-    <mergeCell ref="N30:V30"/>
-    <mergeCell ref="J10:V10"/>
-    <mergeCell ref="E41:G41"/>
-    <mergeCell ref="A58:C58"/>
-    <mergeCell ref="E47:G47"/>
-    <mergeCell ref="E43:G43"/>
-    <mergeCell ref="A60:C60"/>
-    <mergeCell ref="F58:V58"/>
-    <mergeCell ref="N32:V32"/>
-    <mergeCell ref="G30:M30"/>
-    <mergeCell ref="H42:L42"/>
-    <mergeCell ref="F60:V60"/>
-    <mergeCell ref="M46:V46"/>
-    <mergeCell ref="F57:V57"/>
-    <mergeCell ref="M42:V42"/>
-    <mergeCell ref="M3:V3"/>
-    <mergeCell ref="N33:V33"/>
-    <mergeCell ref="G3:I3"/>
-    <mergeCell ref="J4:L4"/>
-    <mergeCell ref="J12:V12"/>
-    <mergeCell ref="A53:V53"/>
-    <mergeCell ref="G32:M32"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="E45:G45"/>
-    <mergeCell ref="M4:V4"/>
-    <mergeCell ref="H46:L46"/>
-    <mergeCell ref="G2:J2"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="E31:F31"/>
-    <mergeCell ref="M44:V44"/>
-    <mergeCell ref="Q2:V2"/>
-    <mergeCell ref="H45:L45"/>
-    <mergeCell ref="A1:V1"/>
-    <mergeCell ref="M51:V51"/>
-    <mergeCell ref="A59:C59"/>
-    <mergeCell ref="H47:L47"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="D55:E55"/>
-    <mergeCell ref="F56:V56"/>
-    <mergeCell ref="E32:F32"/>
-    <mergeCell ref="A37:V37"/>
-    <mergeCell ref="D54:E54"/>
-    <mergeCell ref="J11:V11"/>
-    <mergeCell ref="E51:G51"/>
-    <mergeCell ref="A54:C54"/>
-    <mergeCell ref="M45:V45"/>
-    <mergeCell ref="E33:F33"/>
-    <mergeCell ref="A56:C56"/>
-    <mergeCell ref="A27:C27"/>
-    <mergeCell ref="H50:L50"/>
-    <mergeCell ref="F54:V54"/>
-    <mergeCell ref="M47:V47"/>
-    <mergeCell ref="E35:F35"/>
-    <mergeCell ref="G31:M31"/>
-    <mergeCell ref="K2:M2"/>
-    <mergeCell ref="H39:L39"/>
-    <mergeCell ref="E49:G49"/>
-    <mergeCell ref="M50:V50"/>
-    <mergeCell ref="D57:E57"/>
-    <mergeCell ref="J7:V7"/>
-    <mergeCell ref="N34:V34"/>
-    <mergeCell ref="M49:V49"/>
-    <mergeCell ref="E30:F30"/>
-    <mergeCell ref="J13:V13"/>
-    <mergeCell ref="A6:V6"/>
-    <mergeCell ref="E50:G50"/>
-    <mergeCell ref="D58:E58"/>
-    <mergeCell ref="M40:V40"/>
-    <mergeCell ref="E39:G39"/>
-    <mergeCell ref="E48:G48"/>
-    <mergeCell ref="G34:M34"/>
-    <mergeCell ref="D59:E59"/>
-    <mergeCell ref="E38:G38"/>
-  </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId2"/>
@@ -5057,7 +4408,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H28"/>
+  <dimension ref="A1:I28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5076,55 +4427,53 @@
           <t>💸 ДИАГНОСТИЧЕСКИЙ АУДИТ УПУЩЕННОЙ ПРИБЫЛИ И УЗКИХ МЕСТ ОТДЕЛА ПРОДАЖ</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
     </row>
     <row r="2" ht="24" customHeight="1">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>⚡ Экспресс-Калькулятор</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="n"/>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>📋 Пульт РОПа</t>
-        </is>
-      </c>
-      <c r="D2" s="4" t="inlineStr">
-        <is>
-          <t>🎙️ ИИ-Аудит</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="inlineStr">
-        <is>
-          <t>💸 7 Грехов ОП</t>
-        </is>
-      </c>
-      <c r="F2" s="4" t="inlineStr">
-        <is>
-          <t>📄 One-Pager</t>
-        </is>
-      </c>
-      <c r="G2" s="4" t="inlineStr">
-        <is>
-          <t>🔐 152-ФЗ Безопасность</t>
-        </is>
-      </c>
-      <c r="H2" s="4" t="n"/>
-    </row>
+      <c r="A2" s="133">
+        <f>HYPERLINK("#'📄 Executive_OnePager'!A1", "📄 1. One-Pager")</f>
+        <v/>
+      </c>
+      <c r="B2" s="133">
+        <f>HYPERLINK("#'⚡ Пульс_Компании'!A1", "⚡ 2. Пульс компании")</f>
+        <v/>
+      </c>
+      <c r="C2" s="133">
+        <f>HYPERLINK("#'📋 Пульт_РОПа_15_Минут'!A1", "📋 3. Пульт РОПа")</f>
+        <v/>
+      </c>
+      <c r="D2" s="133">
+        <f>HYPERLINK("#'💸 Диагностика_Утечек_ОП'!A1", "💸 4. 7 Грехов ОП")</f>
+        <v/>
+      </c>
+      <c r="E2" s="133">
+        <f>HYPERLINK("#'🎯 Action_Center'!A1", "🎯 5. Action Center")</f>
+        <v/>
+      </c>
+      <c r="F2" s="133">
+        <f>HYPERLINK("#'🎙️ ИИ_Аудит'!A1", "🎙️ 6. ИИ-Аудит")</f>
+        <v/>
+      </c>
+      <c r="G2" s="133">
+        <f>HYPERLINK("#'⚡ Экспресс_Калькулятор_3_Цифры'!A1", "⚡ 7. Экспресс 3 цифры")</f>
+        <v/>
+      </c>
+      <c r="H2" s="133">
+        <f>HYPERLINK("#'🧪 QA_Suite'!A1", "🧪 8. QA Suite")</f>
+        <v/>
+      </c>
+      <c r="I2" s="133">
+        <f>HYPERLINK("#'⚙️ Настройки'!A1", "⚙️ 9. Настройки")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="39" t="inlineStr">
         <is>
           <t>Фактическая выручка месяца</t>
         </is>
       </c>
-      <c r="B4" s="39" t="n"/>
+      <c r="B4" s="98" t="n"/>
       <c r="C4" s="53" t="inlineStr">
         <is>
           <t>Взвешенный пайплайн в работе</t>
@@ -5150,13 +4499,13 @@
           <t>Срок окупаемости проекта</t>
         </is>
       </c>
-      <c r="H4" s="85" t="n"/>
+      <c r="H4" s="98" t="n"/>
     </row>
     <row r="5" ht="32" customHeight="1">
       <c r="A5" s="86" t="n">
         <v>1650000</v>
       </c>
-      <c r="B5" s="86" t="n"/>
+      <c r="B5" s="98" t="n"/>
       <c r="C5" s="23" t="n">
         <v>2754000</v>
       </c>
@@ -5176,8 +4525,9 @@
           <t>6 дн.</t>
         </is>
       </c>
-      <c r="H5" s="87" t="n"/>
-    </row>
+      <c r="H5" s="98" t="n"/>
+    </row>
+    <row r="6"/>
     <row r="7" ht="24" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
@@ -5525,6 +4875,7 @@
         </is>
       </c>
     </row>
+    <row r="17"/>
     <row r="18" ht="26" customHeight="1">
       <c r="A18" s="50" t="inlineStr">
         <is>
@@ -5555,8 +4906,8 @@
           <t>Стоимость проекта оптимизации ОП</t>
         </is>
       </c>
-      <c r="B20" s="51" t="n"/>
-      <c r="C20" s="51" t="n"/>
+      <c r="B20" s="99" t="n"/>
+      <c r="C20" s="98" t="n"/>
       <c r="D20" s="83" t="n">
         <v>450000</v>
       </c>
@@ -5565,9 +4916,9 @@
           <t>Фиксированная стоимость внедрения (4 недели спринтов)</t>
         </is>
       </c>
-      <c r="F20" s="51" t="n"/>
-      <c r="G20" s="51" t="n"/>
-      <c r="H20" s="51" t="n"/>
+      <c r="F20" s="99" t="n"/>
+      <c r="G20" s="99" t="n"/>
+      <c r="H20" s="98" t="n"/>
     </row>
     <row r="21" ht="22" customHeight="1">
       <c r="A21" s="8" t="inlineStr">
@@ -5575,8 +4926,8 @@
           <t>Ожидаемый возврат выручки (M1 факт)</t>
         </is>
       </c>
-      <c r="B21" s="51" t="n"/>
-      <c r="C21" s="51" t="n"/>
+      <c r="B21" s="99" t="n"/>
+      <c r="C21" s="98" t="n"/>
       <c r="D21" s="82" t="n">
         <v>2100300</v>
       </c>
@@ -5585,9 +4936,9 @@
           <t>Консервативный ориентир: устранение всего 30% найденных узких мест</t>
         </is>
       </c>
-      <c r="F21" s="51" t="n"/>
-      <c r="G21" s="51" t="n"/>
-      <c r="H21" s="51" t="n"/>
+      <c r="F21" s="99" t="n"/>
+      <c r="G21" s="99" t="n"/>
+      <c r="H21" s="98" t="n"/>
     </row>
     <row r="22" ht="22" customHeight="1">
       <c r="A22" s="8" t="inlineStr">
@@ -5595,8 +4946,8 @@
           <t>Чистая прибыль собственника за вычетом услуг</t>
         </is>
       </c>
-      <c r="B22" s="51" t="n"/>
-      <c r="C22" s="51" t="n"/>
+      <c r="B22" s="99" t="n"/>
+      <c r="C22" s="98" t="n"/>
       <c r="D22" s="82">
         <f>D21-D20</f>
         <v/>
@@ -5606,9 +4957,9 @@
           <t>Чистый денежный плюс в кассе компании в первый же месяц</t>
         </is>
       </c>
-      <c r="F22" s="51" t="n"/>
-      <c r="G22" s="51" t="n"/>
-      <c r="H22" s="51" t="n"/>
+      <c r="F22" s="99" t="n"/>
+      <c r="G22" s="99" t="n"/>
+      <c r="H22" s="98" t="n"/>
     </row>
     <row r="23" ht="22" customHeight="1">
       <c r="A23" s="8" t="inlineStr">
@@ -5616,8 +4967,8 @@
           <t>Чистый ROI инвестиций в проект</t>
         </is>
       </c>
-      <c r="B23" s="51" t="n"/>
-      <c r="C23" s="51" t="n"/>
+      <c r="B23" s="99" t="n"/>
+      <c r="C23" s="98" t="n"/>
       <c r="D23" s="60">
         <f>(D22/D20)*100 &amp; "%"</f>
         <v/>
@@ -5627,9 +4978,9 @@
           <t>Процент отдачи на каждый вложенный рубль</t>
         </is>
       </c>
-      <c r="F23" s="51" t="n"/>
-      <c r="G23" s="51" t="n"/>
-      <c r="H23" s="51" t="n"/>
+      <c r="F23" s="99" t="n"/>
+      <c r="G23" s="99" t="n"/>
+      <c r="H23" s="98" t="n"/>
     </row>
     <row r="24" ht="22" customHeight="1">
       <c r="A24" s="8" t="inlineStr">
@@ -5637,8 +4988,8 @@
           <t>Срок полной окупаемости проекта</t>
         </is>
       </c>
-      <c r="B24" s="51" t="n"/>
-      <c r="C24" s="51" t="n"/>
+      <c r="B24" s="99" t="n"/>
+      <c r="C24" s="98" t="n"/>
       <c r="D24" s="60">
         <f>ROUND(D20/(D21/30), 0) &amp; " дн."</f>
         <v/>
@@ -5648,10 +4999,11 @@
           <t>Количество дней работы ОП до полной окупаемости чека внедрения</t>
         </is>
       </c>
-      <c r="F24" s="51" t="n"/>
-      <c r="G24" s="51" t="n"/>
-      <c r="H24" s="51" t="n"/>
-    </row>
+      <c r="F24" s="99" t="n"/>
+      <c r="G24" s="99" t="n"/>
+      <c r="H24" s="98" t="n"/>
+    </row>
+    <row r="25"/>
     <row r="26" ht="28" customHeight="1">
       <c r="A26" s="92" t="inlineStr">
         <is>
@@ -5674,8 +5026,7 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="25">
-    <mergeCell ref="G2:H2"/>
+  <mergeCells count="23">
     <mergeCell ref="A21:C21"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="E22:H22"/>
@@ -5689,7 +5040,6 @@
     <mergeCell ref="E24:H24"/>
     <mergeCell ref="A18:H18"/>
     <mergeCell ref="A26:H26"/>
-    <mergeCell ref="A2:B2"/>
     <mergeCell ref="A19:C19"/>
     <mergeCell ref="E23:H23"/>
     <mergeCell ref="A5:B5"/>
@@ -5739,50 +5089,46 @@
           <t>📄 REVOPS ENTERPRISE EXECUTIVE ONE-PAGER (УПРАВЛЕНЧЕСКИЙ ДАЙДЖЕСТ)</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
-      <c r="I1" s="2" t="n"/>
     </row>
     <row r="2" ht="24" customHeight="1">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>⚡ Экспресс-Калькулятор</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>📋 Пульт РОПа (15 мин)</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="n"/>
-      <c r="D2" s="4" t="inlineStr">
-        <is>
-          <t>🎙️ ИИ-Аудит звонков</t>
-        </is>
-      </c>
-      <c r="E2" s="4" t="n"/>
-      <c r="F2" s="4" t="inlineStr">
-        <is>
-          <t>💸 7 Грехов (Диагностика)</t>
-        </is>
-      </c>
-      <c r="G2" s="3" t="inlineStr">
-        <is>
-          <t>📄 Executive One-Pager</t>
-        </is>
-      </c>
-      <c r="H2" s="3" t="n"/>
-      <c r="I2" s="4" t="inlineStr">
-        <is>
-          <t>🔐 152-ФЗ Безопасность</t>
-        </is>
-      </c>
-    </row>
+      <c r="A2" s="133">
+        <f>HYPERLINK("#'📄 Executive_OnePager'!A1", "📄 1. One-Pager")</f>
+        <v/>
+      </c>
+      <c r="B2" s="133">
+        <f>HYPERLINK("#'⚡ Пульс_Компании'!A1", "⚡ 2. Пульс компании")</f>
+        <v/>
+      </c>
+      <c r="C2" s="133">
+        <f>HYPERLINK("#'📋 Пульт_РОПа_15_Минут'!A1", "📋 3. Пульт РОПа")</f>
+        <v/>
+      </c>
+      <c r="D2" s="133">
+        <f>HYPERLINK("#'💸 Диагностика_Утечек_ОП'!A1", "💸 4. 7 Грехов ОП")</f>
+        <v/>
+      </c>
+      <c r="E2" s="133">
+        <f>HYPERLINK("#'🎯 Action_Center'!A1", "🎯 5. Action Center")</f>
+        <v/>
+      </c>
+      <c r="F2" s="133">
+        <f>HYPERLINK("#'🎙️ ИИ_Аудит'!A1", "🎙️ 6. ИИ-Аудит")</f>
+        <v/>
+      </c>
+      <c r="G2" s="133">
+        <f>HYPERLINK("#'⚡ Экспресс_Калькулятор_3_Цифры'!A1", "⚡ 7. Экспресс 3 цифры")</f>
+        <v/>
+      </c>
+      <c r="H2" s="133">
+        <f>HYPERLINK("#'🧪 QA_Suite'!A1", "🧪 8. QA Suite")</f>
+        <v/>
+      </c>
+      <c r="I2" s="133">
+        <f>HYPERLINK("#'⚙️ Настройки'!A1", "⚙️ 9. Настройки")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="95" t="inlineStr">
         <is>
@@ -5859,6 +5205,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7" ht="24" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
@@ -6099,26 +5446,24 @@
         <v>0</v>
       </c>
     </row>
+    <row r="15"/>
     <row r="16" ht="32" customHeight="1">
       <c r="A16" s="97" t="inlineStr">
         <is>
           <t>🎯 ГЛАВНЫЙ ФОКУС РУКОВОДСТВА ДО КОНЦА МЕСЯЦА: Перехват сделки D-104 (850 000 ₽) и перераспределение 3 лидов с перегруженного РОПа на КАМов.</t>
         </is>
       </c>
-      <c r="B16" s="97" t="n"/>
-      <c r="C16" s="97" t="n"/>
-      <c r="D16" s="97" t="n"/>
-      <c r="E16" s="97" t="n"/>
-      <c r="F16" s="97" t="n"/>
-      <c r="G16" s="97" t="n"/>
-      <c r="H16" s="97" t="n"/>
-      <c r="I16" s="97" t="n"/>
+      <c r="B16" s="99" t="n"/>
+      <c r="C16" s="99" t="n"/>
+      <c r="D16" s="99" t="n"/>
+      <c r="E16" s="99" t="n"/>
+      <c r="F16" s="99" t="n"/>
+      <c r="G16" s="99" t="n"/>
+      <c r="H16" s="99" t="n"/>
+      <c r="I16" s="98" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="G2:H2"/>
+  <mergeCells count="4">
     <mergeCell ref="F7:I7"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A7:D7"/>
@@ -6159,11 +5504,6 @@
           <t>🔐 ЮРИДИЧЕСКИЙ КОНТУР БЕЗОПАСНОСТИ И ОБЕЗЛИЧИВАНИЯ ПДН (152-ФЗ РФ)</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
     </row>
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="4" t="inlineStr">
@@ -6197,6 +5537,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="24" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
         <is>

</xml_diff>